<commit_message>
not just two size bins
the model variable setup can deal with the situation where the model is to be setup with more particle size bins than was present in the outdoor simulation (in addition to the same number as it could do before)
</commit_message>
<xml_diff>
--- a/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
+++ b/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Documents/GitHub/NCAS-BoxModellingToolkit/indoor_environment_PyCHAM_setup/src/indoor_environment_PyCHAM_setup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4E22B8-9761-2B4B-9179-DD6B49E14C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63E5A6B-FED0-9348-BDAA-8DBBD09655F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="620" yWindow="3700" windowWidth="35500" windowHeight="16600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5760" yWindow="5900" windowWidth="31060" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_emi" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="201">
   <si>
     <t>ACRYLONITRILE</t>
   </si>
@@ -449,9 +449,6 @@
     <t>myosmine</t>
   </si>
   <si>
-    <t>Frying (these values represent particles/ or molecules/s/person/meal or mole fraction of particles; particles from 10.1016/j.atmosenv.2010.01.009, using Table 2, which gives units in /min, and so /60 to convert to /s, e.g. 8.02e12 particles/60, gases from https://onlinelibrary.wiley.com/doi/full/10.1111/ina.12906 (Table 4), assuming stir fry lasted 15 minutes, e.g. for ethanol from table 4: ((67.e-3/46.0684)*6.022e23)/(15.*60.), note that citral not in MCM, so represented by limonene).  Particle radius of 0.05 um is the median average particle size when weighted by number concentration in figure 24 of this reference. Black carbon to primary organic mole fractions estimated from Table 18 of http://dx.doi.org/10.1016/j.atmosenv.2013.01.061</t>
-  </si>
-  <si>
     <t>bleach cleaning using Table 2 of https://onlinelibrary.wiley.com/doi/full/10.1111/ina.12906  and assuming cleaning lasts 15 minutes, e.g. for methanol from table 2: ((1.06e-3/32.0419)*6.022e23)/(15.*60.) note that the chloroamines are not included in the MCM, so were omitted</t>
   </si>
   <si>
@@ -491,9 +488,6 @@
     <t>silicon dioxide from indoors</t>
   </si>
   <si>
-    <t>in Table 1 they give the mass fraction of PM10 that is PM2.5 and they give the number of PM10  particles emitted/min emission rate, whilst their Figure  3 indicates that particle number concentration for washable filter bag less vacuum is dominated by PM2.5 (with a mean radius around 0.015 um), which is consistent with Figure 14 of doi.org/10.1016/j.atmosenv.2010.01.009. To get emission rate of PM2.5 particles in number/unit of time, first multiply the mass emission rate of PM10 (ug/s) from their Table 1 by 0.742 (the mass fraction that is PM2.5 from their Table 1), giving 0.93492 ug/s, then get mass of one particle of radius 0.015 um (radius set for vacuum cleaning for PM0 in indoor_emi sheet of this file), assuming a density of 1.4e-6 ug/um3, giving (using mass emission rate of PM10 (ug/s) from the washable filter bag less vacuum in their Table 1): (0.742*1.26)/((4./3.)*np.pi*0.015**3*1.4e-6) = 4.7e10 particles/s of PM2.5 with a mean radius of 0.015 um, likewise, the same can be done for PM2.5-PM10 assuming a mean radius of 2.5 um: ((1.-0.742)*1.26)/((4./3.)*np.pi*2.5**3*1.4e-6) = 3.5e3 particles/s of PM2.5-PM10 with a mean radius of 2.5 um</t>
-  </si>
-  <si>
     <t>nalk_ind_pm0</t>
   </si>
   <si>
@@ -518,9 +512,6 @@
     <t>wood burning stove PM needs updating to Table 4 of https://doi.org/10.1016/j.jobe.2023.107848 (Table 5 of 10.1021/es00161a010), for carbon monoxide (which is given as cm3/h), molar volume (mol/cm3) found using gas-phase density from Wikipedia (1.145e-3 g/cm3) and molar mass (28.010 g/mol), this then multiplied by value in Table V to give mol/h, followed by conversion to molecules/s, the whole equation is (using a mean average of 70 cm3/h from airtight stoves): 70*(1.145e-3/28.010)*6.022e23/3.6e3; for PM1, mg/h converted to particles/s by dividing by mass of one particle of radius 50 nm and density 1.8 g/cm3 (assuming made of black carbon and using density from AeroMix description paper in GMD), and dividing by 60 to convert /min to /s, the whole equation (using the mean TSP (mg/h) from airtight stoves): 4.47e-3/((4./3.)*np.pi*50.e-7**3*1.8)/3600.; for BaP (which is given in ug/h) converted to molecules/cm3/s using the mean average from all airtight stoves: 0.14e-6/252.316*6.022e23/3600.</t>
   </si>
   <si>
-    <t>Smoking Cigarettes (PM: table 2 of 10.1016/j.atmosenv.2010.01.009,  which has units of /min, so /60 to convert to /s (8.83e12/60)), Gases: Table 3 of doi.org/10.1021/es011058w in which ug/cigarette converted to molececules/s/cigarette assuming a cigarette is smoked in 10 minutes), and values taken from the lowest air change rate in Table 3 for a wallboard only room at the lowest air change rate, as these conditions are closest to minimising losses, then the full equation, e.g. for butadiene is: (((350e-6/54.0904)*si.N_A)/(10*60.)). need a reference (and possibly updated values) for particle-phase mole fractions</t>
-  </si>
-  <si>
     <t>candle burning (same ref as smoking) (doi.org/10.1016/j.atmosenv.2010.01.009)</t>
   </si>
   <si>
@@ -531,9 +522,6 @@
   </si>
   <si>
     <t>BZK_ind_pm1</t>
-  </si>
-  <si>
-    <t>page 660 of https://doi.org/10.1080/15459624.2019.1643466 says the mass fraction of cleaning spray emitted on a single spray that goes airbourne (as gas and particles) rather than deposit on the surface to be cleaned is up to 1/3 (backed up by Figure S5 of https://doi.org/10.1016/j.ijheh.2023.114220), also mass of airbourne particles from cleaning spray is small (maximum mass fraction compared to airbourne particles+gas is 0.01%) compared to gas-phase from cleaning spray. Article https://doi.org/10.1016/j.ijheh.2023.114220 says the average emission rate (of total material (airbourne+deposited) is 1.6 g/s of cleaning spray). Suggest the following: convert the size-resolved plots of particle in the paper (Fig. 3 which suggests that the ratio in PM2.5 to PM10 is about 50:50) into an emission rate of particle containing a non-volatile material, and convert the mass of VOC released into individual components based on a mass-weighted ingredient list. This website (https://www.statista.com/statistics/304000/leading-brands-of-household-cleaners-in-the-uk/) suggests Dettol anti-bacterial surface cleanser is one of the best selling in the UK. The back of the dettol bottle lists: benzalkonium chloride as 0.096 % by mass, then there is also an unamed fragrance, sodium bicarbonate, sodium carbonate, sodium edetate, water, C9-C11 alkylpolyglycoside and C12-C16 Pareth-7. I think I can use this article (https://doi.org/10.1039/D2EA00054G) to get the VOC emission rates for commercial cleaning products, and the same article indicates that benzalkonium chloride is non-volatile, so this along with the sodium salts could represent the non-volatile particles</t>
   </si>
   <si>
     <t>Source and Emission Rate (particle/s or molecules/s or mole fractions for particle components)</t>
@@ -587,9 +575,6 @@
     <t>ALLYLAMINE</t>
   </si>
   <si>
-    <t>cleaning spray (https://doi.org/10.1016/j.ijheh.2023.114220 says that the average total mass emission of material from a spray bottle is 1.6 g/s, whilst both the same article and https://doi.org/10.1080/15459624.2019.1643466 say that up to 1/3 of the sprayed material goes airbourne, and the latter study says up to 0.01 % of the airbourne material is particle rather than gas. Therefore, assuming a particle density of 1g/cm^3 and given that Fig. 3 of the latter paper indicates the particle mass is split roughly evenly between PM2.5 and PM10, and assuming a mean radius of the PM2.5 of 1 um and mean radius of the PM10 of 2 um, the equation for pconc in PM2.5 is: (0.0001*(1.6*1./3.)*0.5)/(4./3.*np.pi*1.e-4**3*1.) , whilst for PM10 it is: 0.0001*(1.6*1./3.)*0.5)/(4./3.*np.pi*2.5e-4**3*1.)), and see notes in cleaning_spray_notes sheet for reasoning behind particle composition. Then, rate of VOC emission is given by combining the previously mentioned total emission mass of gas-phase material with mass fractions given in Table 1 of https://doi.org/10.1039/D2EA00054G, e.g. for allylamine ((0.9999*(1.6*1./3.))*0.003e-3/57.09*si.N_A), limonene emission rate based on average factor for general purpose cleaning products (GPC) in Table 6 of  https://doi.org/10.1111/j.1600-0668.2005.00414.x and converted to molecules/s by: (1.6)*10.e-3/136.23*si.N_A</t>
-  </si>
-  <si>
     <t>HEX1ENE</t>
   </si>
   <si>
@@ -613,12 +598,57 @@
   <si>
     <t xml:space="preserve">used as a replacememt for linalool and bornyl acetate, which are not in the MCM, and as a representative of monoterpene alcohols which are reported in natural product mopping emissions </t>
   </si>
+  <si>
+    <t>Smoking Cigarettes (PM: table 2 (particle number) and Fig. 19 (radius) of 10.1016/j.atmosenv.2010.01.009,  which has units of /min, so /60 to convert to /s (8.83e12/60)), Gases: Table 3 of doi.org/10.1021/es011058w in which ug/cigarette converted to molececules/s/cigarette assuming a cigarette is smoked in 10 minutes), and values taken from the lowest air change rate in Table 3 for a wallboard only room at the lowest air change rate, as these conditions are closest to minimising losses, then the full equation, e.g. for butadiene is: (((350e-6/54.0904)*si.N_A)/(10*60.)). need a reference (and possibly updated values) for particle-phase mole fractions</t>
+  </si>
+  <si>
+    <t>in Table 1 they give the mass fraction of PM10 that is PM2.5 and they give the number of PM10  particles emitted/min emission rate, whilst their Figure  3 indicates that particle number concentration for washable filter bag less vacuum is dominated by PM2.5 (with a mean radius around 0.015 um), which is consistent with Figure 14 of doi.org/10.1016/j.atmosenv.2010.01.009. To get emission rate of PM2.5 particles in number/unit of time, first multiply the mass emission rate of PM10 (ug/s) from their Table 1 by 0.742 (the mass fraction that is PM2.5 from their Table 1), giving 0.93492 ug/s, then get mass of one particle of radius 0.015 um (radius set for vacuum cleaning for PM2.5 in indoor_emi sheet of this file), assuming a density of 1.4e-6 ug/um3, giving (using mass emission rate of PM10 (ug/s) from the washable filter bag less vacuum in their Table 1): (0.742*1.26)/((4./3.)*np.pi*0.015**3*1.4e-6) = 4.7e10 particles/s of PM2.5 with a mean radius of 0.015 um, likewise, the same can be done for PM2.5-PM10 assuming a mean radius of 2.5 um: ((1.-0.742)*1.26)/((4./3.)*np.pi*2.5**3*1.4e-6) = 3.5e3 particles/s of PM2.5-PM10 with a mean radius of 2.5 um</t>
+  </si>
+  <si>
+    <t>Frying (these values represent particles/ or molecules/s/person/meal or mole fraction of particles; particles from 10.1016/j.atmosenv.2010.01.009, using Table 2, which gives units in /min, and so /60 to convert to /s, e.g. 8.02e12 particles/60, gases from https://onlinelibrary.wiley.com/doi/full/10.1111/ina.12906 (Table 4), assuming stir fry lasted 15 minutes, e.g. for ethanol from table 4: ((67.e-3/46.0684)*6.022e23)/(15.*60.), note that citral not in MCM, so represented by limonene).  Particle radius of 0.03 um is suggested by Figure 12 of this reference. Black carbon to primary organic mole fractions estimated from Table 18 of http://dx.doi.org/10.1016/j.atmosenv.2013.01.061</t>
+  </si>
+  <si>
+    <t>page 660 of https://doi.org/10.1080/15459624.2019.1643466 says the mass fraction of cleaning spray emitted on a single spray that goes airbourne (as gas and particles) rather than deposit on the surface to be cleaned is up to 1/3 (backed up by Figure S5 of https://doi.org/10.1016/j.ijheh.2023.114220), also mass of airbourne particles from cleaning spray is small (maximum mass fraction compared to airbourne particles+gas is 0.01%) compared to gas-phase from cleaning spray. Article https://doi.org/10.1016/j.ijheh.2023.114220 says the average emission rate (of total material (airbourne+deposited) is 1.6 g/s of cleaning spray). Suggest the following: convert the size-resolved plots of particle in the paper (Fig. 3 which suggests that the ratio in PM2.5 to PM10 is about 50:50) into an emission rate of particle containing a non-volatile material, and convert the mass of VOC released into individual components based on a mass-weighted ingredient list. This website (https://www.statista.com/statistics/304000/leading-brands-of-household-cleaners-in-the-uk/) suggests Dettol anti-bacterial surface cleanser is one of the best selling in the UK. The back of the dettol bottle lists: benzalkonium chloride as 0.096 % by mass, then there is also an unamed fragrance, sodium bicarbonate, sodium carbonate, sodium edetate, water, C9-C11 alkylpolyglycoside and C12-C16 Pareth-7. I think I can use this article (https://doi.org/10.1039/D2EA00054G) to get the VOC emission rates for commercial cleaning products, and the same article indicates that benzalkonium chloride is non-volatile (which the girolami techqnique estimates to have a density of 0.86g/cm^3), so this along with the sodium salts could represent the non-volatile particles</t>
+  </si>
+  <si>
+    <t>cleaning spray (https://doi.org/10.1016/j.ijheh.2023.114220 says that the average total mass emission of material from a spray bottle is 1.6 g/s, whilst both the same article and https://doi.org/10.1080/15459624.2019.1643466 say that up to 1/3 of the sprayed material mass goes airbourne, with a minimum around 4 %, and the latter study says up to 0.01 % of the airbourne material is particle rather than gas, but with a minimum of 0.0001 %. Therefore (using values toward the lower end of fractions going airbourne and fractions of that in the particle-phase), given that Fig. 3 of the latter paper indicates the particle mass is split roughly evenly between PM2.5 and PM10, and assuming a mean radius of the PM2.5 of 1 um and mean radius of the PM10 of 2.5 um, and knowing that the girolami estimation gives a density for BZK of 0.86 g/cm^-3, the equation for pconc in PM2.5 is: (0.0001*(1.6*1./10.)*0.5)/(4./3.*np.pi*1.e-4**3*0.86) , whilst for PM10 it is: (0.0001*(1.6*1./10.)*0.5)/(4./3.*np.pi*2.5e-4**3*0.86), and see notes in cleaning_spray_notes sheet for reasoning behind particle composition. Then, rate of VOC emission is given by combining the previously mentioned total emission mass of gas-phase material with mass fractions given in Table 1 of https://doi.org/10.1039/D2EA00054G, e.g. for allylamine ((0.9999*(1.6*1./10.))*0.003e-3/57.09*si.N_A), limonene emission rate based on average factor for general purpose cleaning products (GPC) in Table 6 of  https://doi.org/10.1111/j.1600-0668.2005.00414.x (typical value around 15mg/g product) and converted to molecules/s by: (0.9999*(1.6*1./10.))*15.e-3/136.23*si.N_A</t>
+  </si>
+  <si>
+    <t>pconc_pm2</t>
+  </si>
+  <si>
+    <t>bcin_pm2</t>
+  </si>
+  <si>
+    <t>nalk_ind_pm2</t>
+  </si>
+  <si>
+    <t>SiO2_ind_pm2</t>
+  </si>
+  <si>
+    <t>BZK_ind_pm2</t>
+  </si>
+  <si>
+    <t>PNNCATCOOH_pm2</t>
+  </si>
+  <si>
+    <t>C1213OH_pm2</t>
+  </si>
+  <si>
+    <t>NLIMOOH_pm2</t>
+  </si>
+  <si>
+    <t>CO25C6CHO_pm2</t>
+  </si>
+  <si>
+    <t>mean_rad_pm2</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -639,6 +669,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Menlo"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -682,7 +718,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -691,6 +727,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
@@ -710,6 +747,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -994,7 +1032,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P10108"/>
+  <dimension ref="A1:P10118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -1014,79 +1052,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="6"/>
-      <c r="B1" s="6"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="8"/>
+      <c r="A1" s="7"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="9"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="F2" s="8" t="s">
+      <c r="E2" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="K2" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="I2" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="O2" s="8" t="s">
+      <c r="L2" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="N2" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="O2" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="P2" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="P2" s="8" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="12" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C3" s="10">
-        <v>0</v>
-      </c>
-      <c r="D3" s="10">
+        <v>146</v>
+      </c>
+      <c r="C3" s="11">
+        <v>0</v>
+      </c>
+      <c r="D3" s="11">
         <v>0</v>
       </c>
       <c r="E3">
@@ -1095,37 +1133,39 @@
       <c r="F3">
         <v>133666666666.7</v>
       </c>
-      <c r="G3" s="8">
-        <v>0</v>
-      </c>
-      <c r="H3" s="8">
-        <v>0</v>
-      </c>
-      <c r="I3" s="8">
-        <v>0</v>
-      </c>
-      <c r="J3" s="8">
+      <c r="G3" s="9">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9">
+        <v>0</v>
+      </c>
+      <c r="I3" s="9">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9">
         <v>1317449251.0999999</v>
       </c>
-      <c r="K3" s="8">
-        <v>0</v>
-      </c>
-      <c r="L3" s="12">
+      <c r="K3" s="9">
+        <v>0</v>
+      </c>
+      <c r="L3" s="13">
         <v>47000000000</v>
       </c>
-      <c r="M3">
-        <v>6366197.7236758098</v>
-      </c>
-      <c r="N3" s="8">
-        <v>0</v>
-      </c>
+      <c r="M3" s="6">
+        <v>0</v>
+      </c>
+      <c r="N3" s="9">
+        <v>0</v>
+      </c>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C4" s="4">
         <v>12.010999999999999</v>
@@ -1163,13 +1203,15 @@
       <c r="N4">
         <v>0</v>
       </c>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C5">
         <v>256.42</v>
@@ -1207,13 +1249,15 @@
       <c r="N5">
         <v>0</v>
       </c>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C6" s="4">
         <v>60.084299999999999</v>
@@ -1251,13 +1295,15 @@
       <c r="N6">
         <v>0</v>
       </c>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C7">
         <v>368.03928000000002</v>
@@ -1290,11 +1336,13 @@
         <v>0</v>
       </c>
       <c r="M7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N7">
         <v>0</v>
       </c>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
@@ -1337,6 +1385,8 @@
       <c r="N8">
         <v>0</v>
       </c>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
@@ -1379,6 +1429,8 @@
       <c r="N9">
         <v>0</v>
       </c>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
@@ -1421,6 +1473,8 @@
       <c r="N10">
         <v>0</v>
       </c>
+      <c r="O10" s="9"/>
+      <c r="P10" s="9"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
@@ -1463,22 +1517,24 @@
       <c r="N11">
         <v>0</v>
       </c>
+      <c r="O11" s="9"/>
+      <c r="P11" s="9"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>62</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D12" s="4">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>0.3</v>
+        <v>3.9E-2</v>
       </c>
       <c r="F12">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1499,23 +1555,25 @@
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12">
         <v>0</v>
       </c>
+      <c r="O12" s="9"/>
+      <c r="P12" s="9"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="12" t="s">
         <v>52</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C13" s="4">
-        <v>0</v>
-      </c>
-      <c r="D13" s="4">
+        <v>146</v>
+      </c>
+      <c r="C13" s="11">
+        <v>0</v>
+      </c>
+      <c r="D13" s="11">
         <v>0</v>
       </c>
       <c r="E13">
@@ -1524,37 +1582,37 @@
       <c r="F13">
         <v>0</v>
       </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13" s="12">
-        <v>3500</v>
-      </c>
-      <c r="M13">
-        <v>407436.65431525197</v>
-      </c>
-      <c r="N13">
+      <c r="G13" s="9">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9">
+        <v>0</v>
+      </c>
+      <c r="I13" s="9">
+        <v>0</v>
+      </c>
+      <c r="J13" s="9">
+        <v>0</v>
+      </c>
+      <c r="K13" s="9">
+        <v>0</v>
+      </c>
+      <c r="L13" s="13">
+        <v>0</v>
+      </c>
+      <c r="M13" s="6">
+        <v>2220766.6477938802</v>
+      </c>
+      <c r="N13" s="9">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="3" t="s">
         <v>65</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C14" s="4">
         <v>12.010999999999999</v>
@@ -1563,10 +1621,10 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>9.0899999999999995E-2</v>
+        <v>0</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1595,10 +1653,10 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C15">
         <v>256.42</v>
@@ -1628,7 +1686,7 @@
         <v>0</v>
       </c>
       <c r="L15">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M15">
         <v>0</v>
@@ -1639,10 +1697,10 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C16" s="4">
         <v>60.084299999999999</v>
@@ -1672,7 +1730,7 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="M16">
         <v>0</v>
@@ -1683,10 +1741,10 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C17">
         <v>368.03928000000002</v>
@@ -1782,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="F19">
-        <v>0.18634239288307916</v>
+        <v>0</v>
       </c>
       <c r="G19">
         <v>0</v>
@@ -1824,7 +1882,7 @@
         <v>0</v>
       </c>
       <c r="F20">
-        <v>0.39348119099491646</v>
+        <v>0</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -1866,7 +1924,7 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>0.32927641612200437</v>
+        <v>0</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -1898,7 +1956,7 @@
         <v>63</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D22" s="4">
         <v>0</v>
@@ -1907,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="F22">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="G22">
         <v>0</v>
@@ -1925,24 +1983,24 @@
         <v>0</v>
       </c>
       <c r="L22">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="M22">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="N22">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>54</v>
+      <c r="A23" s="12" t="s">
+        <v>191</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>55</v>
+        <v>146</v>
       </c>
       <c r="C23" s="4">
-        <v>18.015280000000001</v>
+        <v>0</v>
       </c>
       <c r="D23" s="4">
         <v>0</v>
@@ -1968,25 +2026,25 @@
       <c r="K23">
         <v>0</v>
       </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
-      <c r="M23">
-        <v>0</v>
+      <c r="L23" s="13">
+        <v>3500</v>
+      </c>
+      <c r="M23" s="6">
+        <v>142129.06545880801</v>
       </c>
       <c r="N23">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
-        <v>38</v>
+      <c r="A24" s="12" t="s">
+        <v>192</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C24" s="4">
-        <v>46.025399999999998</v>
+        <v>12.010999999999999</v>
       </c>
       <c r="D24" s="4">
         <v>0</v>
@@ -1995,16 +2053,16 @@
         <v>0</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>9.0899999999999995E-2</v>
       </c>
       <c r="G24">
-        <v>5088253201251670</v>
+        <v>0</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
-      <c r="I24" s="12">
-        <v>7.4580997301490002E+18</v>
+      <c r="I24">
+        <v>0</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -2024,13 +2082,13 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>40</v>
+        <v>193</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" s="4">
-        <v>119.3776</v>
+        <v>150</v>
+      </c>
+      <c r="C25">
+        <v>256.42</v>
       </c>
       <c r="D25" s="4">
         <v>0</v>
@@ -2042,7 +2100,7 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>1289149350929780</v>
+        <v>0</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -2057,7 +2115,7 @@
         <v>0</v>
       </c>
       <c r="L25">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M25">
         <v>0</v>
@@ -2068,13 +2126,13 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>23</v>
+        <v>194</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>24</v>
+        <v>148</v>
       </c>
       <c r="C26" s="4">
-        <v>46.068399999999997</v>
+        <v>60.084299999999999</v>
       </c>
       <c r="D26" s="4">
         <v>0</v>
@@ -2082,8 +2140,8 @@
       <c r="E26">
         <v>0</v>
       </c>
-      <c r="F26" s="12">
-        <v>9.7312788037883699E+17</v>
+      <c r="F26">
+        <v>0</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -2091,17 +2149,17 @@
       <c r="H26">
         <v>0</v>
       </c>
-      <c r="I26" s="12">
-        <v>5.8707519291711396E+21</v>
+      <c r="I26">
+        <v>0</v>
       </c>
       <c r="J26">
         <v>0</v>
       </c>
       <c r="K26">
-        <v>4771231473200710</v>
+        <v>0</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="M26">
         <v>0</v>
@@ -2112,13 +2170,13 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>25</v>
+        <v>195</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="4">
-        <v>32.041899999999998</v>
+        <v>158</v>
+      </c>
+      <c r="C27">
+        <v>368.03928000000002</v>
       </c>
       <c r="D27" s="4">
         <v>0</v>
@@ -2126,11 +2184,11 @@
       <c r="E27">
         <v>0</v>
       </c>
-      <c r="F27" s="12">
-        <v>8.9794231234033504E+16</v>
-      </c>
-      <c r="G27" s="12">
-        <v>2.2135322118157E+16</v>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
       </c>
       <c r="H27">
         <v>0</v>
@@ -2148,7 +2206,7 @@
         <v>0</v>
       </c>
       <c r="M27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -2156,13 +2214,11 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C28" s="4">
-        <v>60.052</v>
+        <v>196</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28">
+        <v>324.19839999999999</v>
       </c>
       <c r="D28" s="4">
         <v>0</v>
@@ -2170,8 +2226,8 @@
       <c r="E28">
         <v>0</v>
       </c>
-      <c r="F28" s="12">
-        <v>3.89976834891242E+16</v>
+      <c r="F28">
+        <v>0</v>
       </c>
       <c r="G28">
         <v>0</v>
@@ -2179,7 +2235,7 @@
       <c r="H28">
         <v>0</v>
       </c>
-      <c r="I28" s="12">
+      <c r="I28">
         <v>0</v>
       </c>
       <c r="J28">
@@ -2200,13 +2256,11 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="4">
-        <v>44.052599999999998</v>
+        <v>197</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29">
+        <v>260.28359999999998</v>
       </c>
       <c r="D29" s="4">
         <v>0</v>
@@ -2214,17 +2268,17 @@
       <c r="E29">
         <v>0</v>
       </c>
-      <c r="F29" s="12">
-        <v>2.56692630577486E+16</v>
-      </c>
-      <c r="G29" s="12">
-        <v>1.57964695739991E+16</v>
+      <c r="F29">
+        <v>0.18634239288307916</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
       </c>
       <c r="H29">
         <v>0</v>
       </c>
-      <c r="I29" s="12">
-        <v>1.7593729219433099E+19</v>
+      <c r="I29">
+        <v>0</v>
       </c>
       <c r="J29">
         <v>0</v>
@@ -2244,13 +2298,11 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C30" s="4">
-        <v>58.079099999999997</v>
+        <v>198</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30">
+        <v>231.2457</v>
       </c>
       <c r="D30" s="4">
         <v>0</v>
@@ -2258,17 +2310,17 @@
       <c r="E30">
         <v>0</v>
       </c>
-      <c r="F30" s="12">
-        <v>1.47464788921009E+16</v>
+      <c r="F30">
+        <v>0.39348119099491646</v>
       </c>
       <c r="G30">
-        <v>8986135574874030</v>
+        <v>0</v>
       </c>
       <c r="H30">
         <v>0</v>
       </c>
-      <c r="I30" s="12">
-        <v>1.88E+19</v>
+      <c r="I30">
+        <v>0</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -2288,13 +2340,11 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" s="4">
-        <v>72.105699999999999</v>
+        <v>199</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31">
+        <v>142.1525</v>
       </c>
       <c r="D31" s="4">
         <v>0</v>
@@ -2303,7 +2353,7 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>4918181071522620</v>
+        <v>0.32927641612200437</v>
       </c>
       <c r="G31">
         <v>0</v>
@@ -2311,7 +2361,7 @@
       <c r="H31">
         <v>0</v>
       </c>
-      <c r="I31" s="12">
+      <c r="I31">
         <v>0</v>
       </c>
       <c r="J31">
@@ -2332,30 +2382,27 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>11</v>
+        <v>200</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C32" s="4">
-        <v>54.090400000000002</v>
+        <v>147</v>
       </c>
       <c r="D32" s="4">
         <v>0</v>
       </c>
-      <c r="E32" s="12">
-        <v>6494526650446900</v>
-      </c>
-      <c r="F32" s="12">
-        <v>0</v>
-      </c>
-      <c r="G32" s="12">
+      <c r="E32">
+        <v>0</v>
+      </c>
+      <c r="F32">
+        <v>2.5</v>
+      </c>
+      <c r="G32">
         <v>0</v>
       </c>
       <c r="H32">
         <v>0</v>
       </c>
-      <c r="I32" s="12">
+      <c r="I32">
         <v>0</v>
       </c>
       <c r="J32">
@@ -2365,10 +2412,10 @@
         <v>0</v>
       </c>
       <c r="L32">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="M32">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -2376,31 +2423,31 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="C33" s="4">
-        <v>68.117000000000004</v>
+        <v>18.015280000000001</v>
       </c>
       <c r="D33" s="4">
         <v>0</v>
       </c>
-      <c r="E33" s="12">
-        <v>4.05206901116216E+16</v>
+      <c r="E33">
+        <v>0</v>
       </c>
       <c r="F33">
-        <v>3438038799255520</v>
-      </c>
-      <c r="G33" s="12">
+        <v>0</v>
+      </c>
+      <c r="G33">
         <v>0</v>
       </c>
       <c r="H33">
         <v>0</v>
       </c>
-      <c r="I33" s="12">
-        <v>2.7450925701073101E+18</v>
+      <c r="I33">
+        <v>0</v>
       </c>
       <c r="J33">
         <v>0</v>
@@ -2420,31 +2467,31 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C34" s="4">
-        <v>56.063299999999998</v>
+        <v>46.025399999999998</v>
       </c>
       <c r="D34" s="4">
         <v>0</v>
       </c>
       <c r="E34">
-        <v>9846540779202550</v>
+        <v>0</v>
       </c>
       <c r="F34">
-        <v>6683556305501490</v>
-      </c>
-      <c r="G34" s="12">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>5088253201251670</v>
       </c>
       <c r="H34">
         <v>0</v>
       </c>
-      <c r="I34" s="12">
-        <v>0</v>
+      <c r="I34" s="13">
+        <v>7.4580997301490002E+18</v>
       </c>
       <c r="J34">
         <v>0</v>
@@ -2464,30 +2511,30 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>115</v>
+        <v>41</v>
       </c>
       <c r="C35" s="4">
-        <v>53.064</v>
+        <v>119.3776</v>
       </c>
       <c r="D35" s="4">
         <v>0</v>
       </c>
       <c r="E35">
-        <v>3612709448841650</v>
+        <v>0</v>
       </c>
       <c r="F35">
         <v>0</v>
       </c>
-      <c r="G35" s="12">
-        <v>0</v>
+      <c r="G35">
+        <v>1289149350929780</v>
       </c>
       <c r="H35">
         <v>0</v>
       </c>
-      <c r="I35" s="12">
+      <c r="I35">
         <v>0</v>
       </c>
       <c r="J35">
@@ -2508,37 +2555,37 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>116</v>
+        <v>24</v>
       </c>
       <c r="C36" s="4">
-        <v>72.105699999999999</v>
+        <v>46.068399999999997</v>
       </c>
       <c r="D36" s="4">
         <v>0</v>
       </c>
       <c r="E36">
-        <v>3855758491862170</v>
-      </c>
-      <c r="F36" s="12">
-        <v>0</v>
-      </c>
-      <c r="G36" s="12">
+        <v>0</v>
+      </c>
+      <c r="F36" s="13">
+        <v>9.7312788037883699E+17</v>
+      </c>
+      <c r="G36">
         <v>0</v>
       </c>
       <c r="H36">
         <v>0</v>
       </c>
-      <c r="I36" s="12">
-        <v>0</v>
+      <c r="I36" s="13">
+        <v>5.8707519291711396E+21</v>
       </c>
       <c r="J36">
         <v>0</v>
       </c>
       <c r="K36">
-        <v>0</v>
+        <v>4771231473200710</v>
       </c>
       <c r="L36">
         <v>0</v>
@@ -2552,30 +2599,30 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>117</v>
+        <v>26</v>
       </c>
       <c r="C37" s="4">
-        <v>41.052999999999997</v>
+        <v>32.041899999999998</v>
       </c>
       <c r="D37" s="4">
         <v>0</v>
       </c>
-      <c r="E37" s="12">
-        <v>2.30306213752953E+16</v>
-      </c>
-      <c r="F37">
-        <v>0</v>
-      </c>
-      <c r="G37" s="12">
-        <v>0</v>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37" s="13">
+        <v>8.9794231234033504E+16</v>
+      </c>
+      <c r="G37" s="13">
+        <v>2.2135322118157E+16</v>
       </c>
       <c r="H37">
         <v>0</v>
       </c>
-      <c r="I37" s="12">
+      <c r="I37">
         <v>0</v>
       </c>
       <c r="J37">
@@ -2596,31 +2643,31 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="C38" s="4">
-        <v>78.111800000000002</v>
+        <v>60.052</v>
       </c>
       <c r="D38" s="4">
         <v>0</v>
       </c>
       <c r="E38">
-        <v>4972719602159980</v>
-      </c>
-      <c r="F38" s="12">
-        <v>0</v>
-      </c>
-      <c r="G38" s="12">
+        <v>0</v>
+      </c>
+      <c r="F38" s="13">
+        <v>3.89976834891242E+16</v>
+      </c>
+      <c r="G38">
         <v>0</v>
       </c>
       <c r="H38">
         <v>0</v>
       </c>
-      <c r="I38" s="12">
-        <v>2.8332937268120801E+18</v>
+      <c r="I38" s="13">
+        <v>0</v>
       </c>
       <c r="J38">
         <v>0</v>
@@ -2631,8 +2678,8 @@
       <c r="L38">
         <v>0</v>
       </c>
-      <c r="M38" s="12">
-        <v>8.6341354134360197E+18</v>
+      <c r="M38">
+        <v>0</v>
       </c>
       <c r="N38">
         <v>0</v>
@@ -2640,31 +2687,31 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>118</v>
+        <v>30</v>
       </c>
       <c r="C39" s="4">
-        <v>92.138400000000004</v>
+        <v>44.052599999999998</v>
       </c>
       <c r="D39" s="4">
         <v>0</v>
       </c>
       <c r="E39">
-        <v>8878029716527880</v>
-      </c>
-      <c r="F39">
-        <v>0</v>
-      </c>
-      <c r="G39" s="12">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F39" s="13">
+        <v>2.56692630577486E+16</v>
+      </c>
+      <c r="G39" s="13">
+        <v>1.57964695739991E+16</v>
       </c>
       <c r="H39">
-        <v>1328950072210210</v>
-      </c>
-      <c r="I39">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="I39" s="13">
+        <v>1.7593729219433099E+19</v>
       </c>
       <c r="J39">
         <v>0</v>
@@ -2684,31 +2731,31 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
       <c r="C40" s="4">
-        <v>106.16500000000001</v>
+        <v>58.079099999999997</v>
       </c>
       <c r="D40" s="4">
         <v>0</v>
       </c>
       <c r="E40">
-        <v>1181757319581150</v>
-      </c>
-      <c r="F40" s="12">
-        <v>0</v>
-      </c>
-      <c r="G40" s="12">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="F40" s="13">
+        <v>1.47464788921009E+16</v>
+      </c>
+      <c r="G40">
+        <v>8986135574874030</v>
       </c>
       <c r="H40">
         <v>0</v>
       </c>
-      <c r="I40" s="12">
-        <v>0</v>
+      <c r="I40" s="13">
+        <v>1.88E+19</v>
       </c>
       <c r="J40">
         <v>0</v>
@@ -2728,30 +2775,30 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>120</v>
+        <v>37</v>
       </c>
       <c r="C41" s="4">
-        <v>106.16500000000001</v>
+        <v>72.105699999999999</v>
       </c>
       <c r="D41" s="4">
         <v>0</v>
       </c>
       <c r="E41">
-        <v>3403461080393720</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>0</v>
-      </c>
-      <c r="G41" s="12">
+        <v>4918181071522620</v>
+      </c>
+      <c r="G41">
         <v>0</v>
       </c>
       <c r="H41">
         <v>0</v>
       </c>
-      <c r="I41" s="12">
+      <c r="I41" s="13">
         <v>0</v>
       </c>
       <c r="J41">
@@ -2772,30 +2819,30 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="C42" s="4">
-        <v>106.16500000000001</v>
+        <v>54.090400000000002</v>
       </c>
       <c r="D42" s="4">
         <v>0</v>
       </c>
-      <c r="E42">
-        <v>671238157522096</v>
-      </c>
-      <c r="F42" s="12">
-        <v>0</v>
-      </c>
-      <c r="G42" s="12">
+      <c r="E42" s="13">
+        <v>6494526650446900</v>
+      </c>
+      <c r="F42" s="13">
+        <v>0</v>
+      </c>
+      <c r="G42" s="13">
         <v>0</v>
       </c>
       <c r="H42">
         <v>0</v>
       </c>
-      <c r="I42" s="12">
+      <c r="I42" s="13">
         <v>0</v>
       </c>
       <c r="J42">
@@ -2816,31 +2863,31 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="C43" s="4">
-        <v>104.1491</v>
+        <v>68.117000000000004</v>
       </c>
       <c r="D43" s="4">
         <v>0</v>
       </c>
-      <c r="E43">
-        <v>1657572670207100</v>
+      <c r="E43" s="13">
+        <v>4.05206901116216E+16</v>
       </c>
       <c r="F43">
-        <v>0</v>
-      </c>
-      <c r="G43" s="12">
+        <v>3438038799255520</v>
+      </c>
+      <c r="G43" s="13">
         <v>0</v>
       </c>
       <c r="H43">
         <v>0</v>
       </c>
-      <c r="I43" s="12">
-        <v>0</v>
+      <c r="I43" s="13">
+        <v>2.7450925701073101E+18</v>
       </c>
       <c r="J43">
         <v>0</v>
@@ -2860,30 +2907,30 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>123</v>
+        <v>35</v>
       </c>
       <c r="C44" s="4">
-        <v>120.19159999999999</v>
+        <v>56.063299999999998</v>
       </c>
       <c r="D44" s="4">
         <v>0</v>
       </c>
       <c r="E44">
-        <v>459291306269878</v>
-      </c>
-      <c r="F44" s="12">
-        <v>0</v>
-      </c>
-      <c r="G44" s="12">
+        <v>9846540779202550</v>
+      </c>
+      <c r="F44">
+        <v>6683556305501490</v>
+      </c>
+      <c r="G44" s="13">
         <v>0</v>
       </c>
       <c r="H44">
         <v>0</v>
       </c>
-      <c r="I44" s="12">
+      <c r="I44" s="13">
         <v>0</v>
       </c>
       <c r="J44">
@@ -2904,30 +2951,30 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="C45" s="4">
-        <v>128.1705</v>
+        <v>53.064</v>
       </c>
       <c r="D45" s="4">
         <v>0</v>
       </c>
       <c r="E45">
-        <v>203603350953092</v>
+        <v>3612709448841650</v>
       </c>
       <c r="F45">
         <v>0</v>
       </c>
-      <c r="G45" s="12">
+      <c r="G45" s="13">
         <v>0</v>
       </c>
       <c r="H45">
         <v>0</v>
       </c>
-      <c r="I45" s="12">
+      <c r="I45" s="13">
         <v>0</v>
       </c>
       <c r="J45">
@@ -2948,30 +2995,30 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="C46" s="4">
-        <v>142.20099999999999</v>
+        <v>72.105699999999999</v>
       </c>
       <c r="D46" s="4">
         <v>0</v>
       </c>
       <c r="E46">
-        <v>115049465648389</v>
-      </c>
-      <c r="F46" s="12">
-        <v>0</v>
-      </c>
-      <c r="G46" s="12">
+        <v>3855758491862170</v>
+      </c>
+      <c r="F46" s="13">
+        <v>0</v>
+      </c>
+      <c r="G46" s="13">
         <v>0</v>
       </c>
       <c r="H46">
         <v>0</v>
       </c>
-      <c r="I46" s="12">
+      <c r="I46" s="13">
         <v>0</v>
       </c>
       <c r="J46">
@@ -2992,30 +3039,30 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="C47" s="4">
-        <v>142.20099999999999</v>
+        <v>41.052999999999997</v>
       </c>
       <c r="D47" s="4">
         <v>0</v>
       </c>
-      <c r="E47">
-        <v>110814515992620</v>
+      <c r="E47" s="13">
+        <v>2.30306213752953E+16</v>
       </c>
       <c r="F47">
         <v>0</v>
       </c>
-      <c r="G47" s="12">
+      <c r="G47" s="13">
         <v>0</v>
       </c>
       <c r="H47">
         <v>0</v>
       </c>
-      <c r="I47" s="12">
+      <c r="I47" s="13">
         <v>0</v>
       </c>
       <c r="J47">
@@ -3036,31 +3083,31 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="C48" s="4">
-        <v>94.111199999999997</v>
+        <v>78.111800000000002</v>
       </c>
       <c r="D48" s="4">
         <v>0</v>
       </c>
       <c r="E48">
-        <v>885189865959984</v>
-      </c>
-      <c r="F48" s="12">
-        <v>0</v>
-      </c>
-      <c r="G48" s="12">
+        <v>4972719602159980</v>
+      </c>
+      <c r="F48" s="13">
+        <v>0</v>
+      </c>
+      <c r="G48" s="13">
         <v>0</v>
       </c>
       <c r="H48">
         <v>0</v>
       </c>
-      <c r="I48" s="12">
-        <v>0</v>
+      <c r="I48" s="13">
+        <v>2.8332937268120801E+18</v>
       </c>
       <c r="J48">
         <v>0</v>
@@ -3071,8 +3118,8 @@
       <c r="L48">
         <v>0</v>
       </c>
-      <c r="M48" s="12">
-        <v>1.3308681516865201E+18</v>
+      <c r="M48" s="14">
+        <v>2.59018093480173E+18</v>
       </c>
       <c r="N48">
         <v>0</v>
@@ -3080,30 +3127,30 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="C49" s="4">
-        <v>108.1378</v>
+        <v>92.138400000000004</v>
       </c>
       <c r="D49" s="4">
         <v>0</v>
       </c>
       <c r="E49">
-        <v>130870341231280</v>
+        <v>8878029716527880</v>
       </c>
       <c r="F49">
         <v>0</v>
       </c>
-      <c r="G49" s="12">
+      <c r="G49" s="13">
         <v>0</v>
       </c>
       <c r="H49">
-        <v>0</v>
-      </c>
-      <c r="I49" s="12">
+        <v>1328950072210210</v>
+      </c>
+      <c r="I49">
         <v>0</v>
       </c>
       <c r="J49">
@@ -3124,30 +3171,30 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>56</v>
+        <v>119</v>
       </c>
       <c r="C50" s="4">
-        <v>108.1378</v>
+        <v>106.16500000000001</v>
       </c>
       <c r="D50" s="4">
         <v>0</v>
       </c>
       <c r="E50">
-        <v>213476443143224</v>
-      </c>
-      <c r="F50" s="12">
-        <v>0</v>
-      </c>
-      <c r="G50" s="12">
+        <v>1181757319581150</v>
+      </c>
+      <c r="F50" s="13">
+        <v>0</v>
+      </c>
+      <c r="G50" s="13">
         <v>0</v>
       </c>
       <c r="H50">
         <v>0</v>
       </c>
-      <c r="I50" s="12">
+      <c r="I50" s="13">
         <v>0</v>
       </c>
       <c r="J50">
@@ -3168,30 +3215,30 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="C51" s="4">
-        <v>79.099999999999994</v>
+        <v>106.16500000000001</v>
       </c>
       <c r="D51" s="4">
         <v>0</v>
       </c>
       <c r="E51">
-        <v>4580684396038760</v>
+        <v>3403461080393720</v>
       </c>
       <c r="F51">
         <v>0</v>
       </c>
-      <c r="G51" s="12">
+      <c r="G51" s="13">
         <v>0</v>
       </c>
       <c r="H51">
         <v>0</v>
       </c>
-      <c r="I51" s="12">
+      <c r="I51" s="13">
         <v>0</v>
       </c>
       <c r="J51">
@@ -3212,30 +3259,30 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="C52" s="4">
-        <v>93.13</v>
+        <v>106.16500000000001</v>
       </c>
       <c r="D52" s="4">
         <v>0</v>
       </c>
       <c r="E52">
-        <v>1422603851820030</v>
-      </c>
-      <c r="F52" s="12">
-        <v>0</v>
-      </c>
-      <c r="G52" s="12">
+        <v>671238157522096</v>
+      </c>
+      <c r="F52" s="13">
+        <v>0</v>
+      </c>
+      <c r="G52" s="13">
         <v>0</v>
       </c>
       <c r="H52">
         <v>0</v>
       </c>
-      <c r="I52" s="12">
+      <c r="I52" s="13">
         <v>0</v>
       </c>
       <c r="J52">
@@ -3256,30 +3303,30 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="C53" s="4">
-        <v>93.13</v>
+        <v>104.1491</v>
       </c>
       <c r="D53" s="4">
         <v>0</v>
       </c>
       <c r="E53">
-        <v>3103862949425530</v>
+        <v>1657572670207100</v>
       </c>
       <c r="F53">
         <v>0</v>
       </c>
-      <c r="G53" s="12">
+      <c r="G53" s="13">
         <v>0</v>
       </c>
       <c r="H53">
         <v>0</v>
       </c>
-      <c r="I53" s="12">
+      <c r="I53" s="13">
         <v>0</v>
       </c>
       <c r="J53">
@@ -3300,30 +3347,30 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C54" s="4">
-        <v>67.09</v>
+        <v>120.19159999999999</v>
       </c>
       <c r="D54" s="4">
         <v>0</v>
       </c>
       <c r="E54">
-        <v>4144017962239770</v>
-      </c>
-      <c r="F54" s="12">
-        <v>0</v>
-      </c>
-      <c r="G54" s="12">
+        <v>459291306269878</v>
+      </c>
+      <c r="F54" s="13">
+        <v>0</v>
+      </c>
+      <c r="G54" s="13">
         <v>0</v>
       </c>
       <c r="H54">
         <v>0</v>
       </c>
-      <c r="I54" s="12">
+      <c r="I54" s="13">
         <v>0</v>
       </c>
       <c r="J54">
@@ -3344,30 +3391,30 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
-        <v>61</v>
+        <v>5</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C55" s="4">
-        <v>105.13720000000001</v>
+        <v>128.1705</v>
       </c>
       <c r="D55" s="4">
         <v>0</v>
       </c>
       <c r="E55">
-        <v>4572763690428630</v>
+        <v>203603350953092</v>
       </c>
       <c r="F55">
         <v>0</v>
       </c>
-      <c r="G55" s="12">
+      <c r="G55" s="13">
         <v>0</v>
       </c>
       <c r="H55">
         <v>0</v>
       </c>
-      <c r="I55" s="12">
+      <c r="I55" s="13">
         <v>0</v>
       </c>
       <c r="J55">
@@ -3388,30 +3435,30 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
-        <v>9</v>
+        <v>57</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C56" s="4">
-        <v>162.23599999999999</v>
+        <v>142.20099999999999</v>
       </c>
       <c r="D56" s="4">
         <v>0</v>
       </c>
       <c r="E56">
-        <v>9898568768132020</v>
-      </c>
-      <c r="F56" s="12">
-        <v>0</v>
-      </c>
-      <c r="G56" s="12">
+        <v>115049465648389</v>
+      </c>
+      <c r="F56" s="13">
+        <v>0</v>
+      </c>
+      <c r="G56" s="13">
         <v>0</v>
       </c>
       <c r="H56">
         <v>0</v>
       </c>
-      <c r="I56" s="12">
+      <c r="I56" s="13">
         <v>0</v>
       </c>
       <c r="J56">
@@ -3432,30 +3479,30 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="C57" s="4">
-        <v>146.19300000000001</v>
+        <v>142.20099999999999</v>
       </c>
       <c r="D57" s="4">
         <v>0</v>
       </c>
       <c r="E57">
-        <v>459989455628290</v>
+        <v>110814515992620</v>
       </c>
       <c r="F57">
         <v>0</v>
       </c>
-      <c r="G57" s="12">
+      <c r="G57" s="13">
         <v>0</v>
       </c>
       <c r="H57">
         <v>0</v>
       </c>
-      <c r="I57" s="12">
+      <c r="I57" s="13">
         <v>0</v>
       </c>
       <c r="J57">
@@ -3476,74 +3523,74 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>34</v>
+        <v>127</v>
       </c>
       <c r="C58" s="4">
-        <v>136.23400000000001</v>
+        <v>94.111199999999997</v>
       </c>
       <c r="D58" s="4">
         <v>0</v>
       </c>
       <c r="E58">
-        <v>0</v>
-      </c>
-      <c r="F58">
-        <v>2996005239351240</v>
-      </c>
-      <c r="G58" s="12">
-        <v>0</v>
-      </c>
-      <c r="H58" s="12">
-        <v>6.13935499867058E+16</v>
-      </c>
-      <c r="I58">
+        <v>885189865959984</v>
+      </c>
+      <c r="F58" s="13">
+        <v>0</v>
+      </c>
+      <c r="G58" s="13">
+        <v>0</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58" s="13">
         <v>0</v>
       </c>
       <c r="J58">
         <v>0</v>
       </c>
       <c r="K58">
-        <v>8929077910066500</v>
+        <v>0</v>
       </c>
       <c r="L58">
         <v>0</v>
       </c>
-      <c r="M58" s="12">
-        <v>7.0729099434779402E+19</v>
+      <c r="M58" s="14">
+        <v>3.9925535458655002E+17</v>
       </c>
       <c r="N58">
-        <v>2343310730695090</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B59" t="s">
-        <v>43</v>
+        <v>18</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="C59" s="4">
-        <v>82.100499999999997</v>
+        <v>108.1378</v>
       </c>
       <c r="D59" s="4">
         <v>0</v>
       </c>
       <c r="E59">
-        <v>0</v>
+        <v>130870341231280</v>
       </c>
       <c r="F59">
         <v>0</v>
       </c>
-      <c r="G59" s="12">
+      <c r="G59" s="13">
         <v>0</v>
       </c>
       <c r="H59">
-        <v>2607968959452810</v>
-      </c>
-      <c r="I59">
+        <v>0</v>
+      </c>
+      <c r="I59" s="13">
         <v>0</v>
       </c>
       <c r="J59">
@@ -3564,30 +3611,30 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="C60" s="4">
-        <v>60.094999999999999</v>
+        <v>108.1378</v>
       </c>
       <c r="D60" s="4">
         <v>0</v>
       </c>
       <c r="E60">
-        <v>0</v>
-      </c>
-      <c r="F60">
-        <v>0</v>
-      </c>
-      <c r="G60" s="12">
+        <v>213476443143224</v>
+      </c>
+      <c r="F60" s="13">
+        <v>0</v>
+      </c>
+      <c r="G60" s="13">
         <v>0</v>
       </c>
       <c r="H60">
         <v>0</v>
       </c>
-      <c r="I60" s="12">
+      <c r="I60" s="13">
         <v>0</v>
       </c>
       <c r="J60">
@@ -3608,34 +3655,34 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
-        <v>46</v>
+        <v>7</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>47</v>
+        <v>129</v>
       </c>
       <c r="C61" s="4">
-        <v>28.01</v>
+        <v>79.099999999999994</v>
       </c>
       <c r="D61" s="4">
         <v>0</v>
       </c>
       <c r="E61">
-        <v>0</v>
+        <v>4580684396038760</v>
       </c>
       <c r="F61">
         <v>0</v>
       </c>
-      <c r="G61" s="12">
+      <c r="G61" s="13">
         <v>0</v>
       </c>
       <c r="H61">
         <v>0</v>
       </c>
-      <c r="I61" s="12">
-        <v>0</v>
-      </c>
-      <c r="J61" s="12">
-        <v>4.7866168828592902E+17</v>
+      <c r="I61" s="13">
+        <v>0</v>
+      </c>
+      <c r="J61">
+        <v>0</v>
       </c>
       <c r="K61">
         <v>0</v>
@@ -3652,34 +3699,34 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>49</v>
+        <v>130</v>
       </c>
       <c r="C62" s="4">
-        <v>252.316</v>
+        <v>93.13</v>
       </c>
       <c r="D62" s="4">
         <v>0</v>
       </c>
       <c r="E62">
-        <v>0</v>
-      </c>
-      <c r="F62">
-        <v>0</v>
-      </c>
-      <c r="G62" s="12">
+        <v>1422603851820030</v>
+      </c>
+      <c r="F62" s="13">
+        <v>0</v>
+      </c>
+      <c r="G62" s="13">
         <v>0</v>
       </c>
       <c r="H62">
         <v>0</v>
       </c>
-      <c r="I62" s="12">
+      <c r="I62" s="13">
         <v>0</v>
       </c>
       <c r="J62">
-        <v>92815710810.606094</v>
+        <v>0</v>
       </c>
       <c r="K62">
         <v>0</v>
@@ -3696,37 +3743,37 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>51</v>
+        <v>131</v>
       </c>
       <c r="C63" s="4">
-        <v>108.1378</v>
+        <v>93.13</v>
       </c>
       <c r="D63" s="4">
         <v>0</v>
       </c>
       <c r="E63">
-        <v>0</v>
+        <v>3103862949425530</v>
       </c>
       <c r="F63">
         <v>0</v>
       </c>
-      <c r="G63" s="12">
+      <c r="G63" s="13">
         <v>0</v>
       </c>
       <c r="H63">
         <v>0</v>
       </c>
-      <c r="I63" s="12">
+      <c r="I63" s="13">
         <v>0</v>
       </c>
       <c r="J63">
         <v>0</v>
       </c>
       <c r="K63">
-        <v>6626896422897450</v>
+        <v>0</v>
       </c>
       <c r="L63">
         <v>0</v>
@@ -3740,31 +3787,31 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
-        <v>96</v>
+        <v>8</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>97</v>
+        <v>132</v>
       </c>
       <c r="C64" s="4">
-        <v>88.148200000000003</v>
+        <v>67.09</v>
       </c>
       <c r="D64" s="4">
         <v>0</v>
       </c>
       <c r="E64">
-        <v>0</v>
-      </c>
-      <c r="F64">
-        <v>0</v>
-      </c>
-      <c r="G64" s="12">
+        <v>4144017962239770</v>
+      </c>
+      <c r="F64" s="13">
+        <v>0</v>
+      </c>
+      <c r="G64" s="13">
         <v>0</v>
       </c>
       <c r="H64">
         <v>0</v>
       </c>
-      <c r="I64" s="12">
-        <v>7.99324851692944E+17</v>
+      <c r="I64" s="13">
+        <v>0</v>
       </c>
       <c r="J64">
         <v>0</v>
@@ -3783,32 +3830,32 @@
       </c>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>98</v>
+      <c r="A65" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C65">
-        <v>76.094399999999993</v>
+        <v>133</v>
+      </c>
+      <c r="C65" s="4">
+        <v>105.13720000000001</v>
       </c>
       <c r="D65" s="4">
         <v>0</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>4572763690428630</v>
       </c>
       <c r="F65">
         <v>0</v>
       </c>
-      <c r="G65" s="12">
+      <c r="G65" s="13">
         <v>0</v>
       </c>
       <c r="H65">
         <v>0</v>
       </c>
-      <c r="I65" s="12">
-        <v>2.8727962844572001E+18</v>
+      <c r="I65" s="13">
+        <v>0</v>
       </c>
       <c r="J65">
         <v>0</v>
@@ -3828,31 +3875,31 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
-        <v>101</v>
+        <v>9</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C66">
-        <v>100.1589</v>
+        <v>134</v>
+      </c>
+      <c r="C66" s="4">
+        <v>162.23599999999999</v>
       </c>
       <c r="D66" s="4">
         <v>0</v>
       </c>
       <c r="E66">
-        <v>0</v>
-      </c>
-      <c r="F66">
-        <v>0</v>
-      </c>
-      <c r="G66" s="12">
+        <v>9898568768132020</v>
+      </c>
+      <c r="F66" s="13">
+        <v>0</v>
+      </c>
+      <c r="G66" s="13">
         <v>0</v>
       </c>
       <c r="H66">
         <v>0</v>
       </c>
-      <c r="I66" s="12">
-        <v>2.1374745930516401E+18</v>
+      <c r="I66" s="13">
+        <v>0</v>
       </c>
       <c r="J66">
         <v>0</v>
@@ -3871,32 +3918,32 @@
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>103</v>
+      <c r="A67" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C67">
-        <v>114.1855</v>
+        <v>135</v>
+      </c>
+      <c r="C67" s="4">
+        <v>146.19300000000001</v>
       </c>
       <c r="D67" s="4">
         <v>0</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>459989455628290</v>
       </c>
       <c r="F67">
         <v>0</v>
       </c>
-      <c r="G67" s="12">
+      <c r="G67" s="13">
         <v>0</v>
       </c>
       <c r="H67">
         <v>0</v>
       </c>
-      <c r="I67" s="12">
-        <v>7.0407870654329997E+17</v>
+      <c r="I67" s="13">
+        <v>0</v>
       </c>
       <c r="J67">
         <v>0</v>
@@ -3916,12 +3963,12 @@
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C68">
+        <v>34</v>
+      </c>
+      <c r="C68" s="4">
         <v>136.23400000000001</v>
       </c>
       <c r="D68" s="4">
@@ -3931,42 +3978,42 @@
         <v>0</v>
       </c>
       <c r="F68">
-        <v>0</v>
-      </c>
-      <c r="G68" s="12">
-        <v>0</v>
-      </c>
-      <c r="H68">
-        <v>0</v>
-      </c>
-      <c r="I68" s="12">
-        <v>3.2841650965559202E+19</v>
+        <v>2996005239351240</v>
+      </c>
+      <c r="G68" s="13">
+        <v>0</v>
+      </c>
+      <c r="H68" s="13">
+        <v>6.13935499867058E+16</v>
+      </c>
+      <c r="I68">
+        <v>0</v>
       </c>
       <c r="J68">
         <v>0</v>
       </c>
       <c r="K68">
-        <v>0</v>
+        <v>8929077910066500</v>
       </c>
       <c r="L68">
         <v>0</v>
       </c>
-      <c r="M68">
-        <v>0</v>
+      <c r="M68" s="14">
+        <v>1.06083039787253E+19</v>
       </c>
       <c r="N68">
-        <v>0</v>
+        <v>2343310730695090</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>107</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="C69">
-        <v>170.24870000000001</v>
+      <c r="A69" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B69" t="s">
+        <v>43</v>
+      </c>
+      <c r="C69" s="4">
+        <v>82.100499999999997</v>
       </c>
       <c r="D69" s="4">
         <v>0</v>
@@ -3977,14 +4024,14 @@
       <c r="F69">
         <v>0</v>
       </c>
-      <c r="G69" s="12">
+      <c r="G69" s="13">
         <v>0</v>
       </c>
       <c r="H69">
-        <v>1375569322343650</v>
-      </c>
-      <c r="I69" s="12">
-        <v>5.9956572873684198E+17</v>
+        <v>2607968959452810</v>
+      </c>
+      <c r="I69">
+        <v>0</v>
       </c>
       <c r="J69">
         <v>0</v>
@@ -3998,19 +4045,19 @@
       <c r="M69">
         <v>0</v>
       </c>
-      <c r="N69" s="12">
-        <v>2.48918362198186E+16</v>
+      <c r="N69">
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>108</v>
+      <c r="A70" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C70">
-        <v>170.24870000000001</v>
+        <v>45</v>
+      </c>
+      <c r="C70" s="4">
+        <v>60.094999999999999</v>
       </c>
       <c r="D70" s="4">
         <v>0</v>
@@ -4021,14 +4068,14 @@
       <c r="F70">
         <v>0</v>
       </c>
-      <c r="G70" s="12">
+      <c r="G70" s="13">
         <v>0</v>
       </c>
       <c r="H70">
         <v>0</v>
       </c>
-      <c r="I70" s="12">
-        <v>4.4569487799906803E+17</v>
+      <c r="I70" s="13">
+        <v>0</v>
       </c>
       <c r="J70">
         <v>0</v>
@@ -4048,13 +4095,13 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
-        <v>110</v>
+        <v>46</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="C71">
-        <v>204.3511</v>
+        <v>47</v>
+      </c>
+      <c r="C71" s="4">
+        <v>28.01</v>
       </c>
       <c r="D71" s="4">
         <v>0</v>
@@ -4065,17 +4112,17 @@
       <c r="F71">
         <v>0</v>
       </c>
-      <c r="G71" s="12">
+      <c r="G71" s="13">
         <v>0</v>
       </c>
       <c r="H71">
         <v>0</v>
       </c>
-      <c r="I71" s="12">
-        <v>5.59185249900783E+18</v>
-      </c>
-      <c r="J71">
-        <v>0</v>
+      <c r="I71" s="13">
+        <v>0</v>
+      </c>
+      <c r="J71" s="13">
+        <v>4.7866168828592902E+17</v>
       </c>
       <c r="K71">
         <v>0</v>
@@ -4092,13 +4139,13 @@
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="B72" t="s">
-        <v>166</v>
-      </c>
-      <c r="C72">
-        <v>57.09</v>
+        <v>48</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C72" s="4">
+        <v>252.316</v>
       </c>
       <c r="D72" s="4">
         <v>0</v>
@@ -4109,17 +4156,17 @@
       <c r="F72">
         <v>0</v>
       </c>
-      <c r="G72" s="12">
+      <c r="G72" s="13">
         <v>0</v>
       </c>
       <c r="H72">
         <v>0</v>
       </c>
-      <c r="I72" s="12">
+      <c r="I72" s="13">
         <v>0</v>
       </c>
       <c r="J72">
-        <v>0</v>
+        <v>92815710810.606094</v>
       </c>
       <c r="K72">
         <v>0</v>
@@ -4127,8 +4174,8 @@
       <c r="L72">
         <v>0</v>
       </c>
-      <c r="M72" s="12">
-        <v>1.68759181528786E+16</v>
+      <c r="M72">
+        <v>0</v>
       </c>
       <c r="N72">
         <v>0</v>
@@ -4136,13 +4183,13 @@
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="B73" t="s">
-        <v>167</v>
-      </c>
-      <c r="C73">
-        <v>76.52</v>
+        <v>50</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C73" s="4">
+        <v>108.1378</v>
       </c>
       <c r="D73" s="4">
         <v>0</v>
@@ -4153,26 +4200,26 @@
       <c r="F73">
         <v>0</v>
       </c>
-      <c r="G73" s="12">
+      <c r="G73" s="13">
         <v>0</v>
       </c>
       <c r="H73">
         <v>0</v>
       </c>
-      <c r="I73" s="12">
+      <c r="I73" s="13">
         <v>0</v>
       </c>
       <c r="J73">
         <v>0</v>
       </c>
       <c r="K73">
-        <v>0</v>
+        <v>6626896422897450</v>
       </c>
       <c r="L73">
         <v>0</v>
       </c>
-      <c r="M73" s="12">
-        <v>6.7150804484951296E+17</v>
+      <c r="M73">
+        <v>0</v>
       </c>
       <c r="N73">
         <v>0</v>
@@ -4180,13 +4227,13 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
-        <v>179</v>
+        <v>96</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="C74">
-        <v>92.52</v>
+        <v>97</v>
+      </c>
+      <c r="C74" s="4">
+        <v>88.148200000000003</v>
       </c>
       <c r="D74" s="4">
         <v>0</v>
@@ -4197,14 +4244,14 @@
       <c r="F74">
         <v>0</v>
       </c>
-      <c r="G74" s="12">
+      <c r="G74" s="13">
         <v>0</v>
       </c>
       <c r="H74">
         <v>0</v>
       </c>
-      <c r="I74" s="12">
-        <v>0</v>
+      <c r="I74" s="13">
+        <v>7.99324851692944E+17</v>
       </c>
       <c r="J74">
         <v>0</v>
@@ -4215,8 +4262,8 @@
       <c r="L74">
         <v>0</v>
       </c>
-      <c r="M74" s="12">
-        <v>2.8116133288360998E+17</v>
+      <c r="M74">
+        <v>0</v>
       </c>
       <c r="N74">
         <v>0</v>
@@ -4224,13 +4271,13 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>169</v>
-      </c>
-      <c r="B75" t="s">
-        <v>170</v>
+        <v>98</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="C75">
-        <v>123.1293</v>
+        <v>76.094399999999993</v>
       </c>
       <c r="D75" s="4">
         <v>0</v>
@@ -4241,14 +4288,14 @@
       <c r="F75">
         <v>0</v>
       </c>
-      <c r="G75" s="12">
+      <c r="G75" s="13">
         <v>0</v>
       </c>
       <c r="H75">
         <v>0</v>
       </c>
-      <c r="I75" s="12">
-        <v>0</v>
+      <c r="I75" s="13">
+        <v>2.8727962844572001E+18</v>
       </c>
       <c r="J75">
         <v>0</v>
@@ -4259,8 +4306,8 @@
       <c r="L75">
         <v>0</v>
       </c>
-      <c r="M75" s="12">
-        <v>3.6515127709569602E+19</v>
+      <c r="M75">
+        <v>0</v>
       </c>
       <c r="N75">
         <v>0</v>
@@ -4268,13 +4315,13 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
-        <v>171</v>
+        <v>101</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>172</v>
+        <v>102</v>
       </c>
       <c r="C76">
-        <v>106.1219</v>
+        <v>100.1589</v>
       </c>
       <c r="D76" s="4">
         <v>0</v>
@@ -4285,14 +4332,14 @@
       <c r="F76">
         <v>0</v>
       </c>
-      <c r="G76" s="12">
+      <c r="G76" s="13">
         <v>0</v>
       </c>
       <c r="H76">
         <v>0</v>
       </c>
-      <c r="I76" s="12">
-        <v>0</v>
+      <c r="I76" s="13">
+        <v>2.1374745930516401E+18</v>
       </c>
       <c r="J76">
         <v>0</v>
@@ -4303,22 +4350,22 @@
       <c r="L76">
         <v>0</v>
       </c>
-      <c r="M76" s="12">
-        <v>6.0524495405619302E+18</v>
+      <c r="M76">
+        <v>0</v>
       </c>
       <c r="N76">
         <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A77" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B77" t="s">
-        <v>174</v>
+      <c r="A77" t="s">
+        <v>103</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="C77">
-        <v>107.15</v>
+        <v>114.1855</v>
       </c>
       <c r="D77" s="4">
         <v>0</v>
@@ -4329,14 +4376,14 @@
       <c r="F77">
         <v>0</v>
       </c>
-      <c r="G77" s="12">
+      <c r="G77" s="13">
         <v>0</v>
       </c>
       <c r="H77">
         <v>0</v>
       </c>
-      <c r="I77" s="12">
-        <v>0</v>
+      <c r="I77" s="13">
+        <v>7.0407870654329997E+17</v>
       </c>
       <c r="J77">
         <v>0</v>
@@ -4347,8 +4394,8 @@
       <c r="L77">
         <v>0</v>
       </c>
-      <c r="M77" s="12">
-        <v>2.2778630803682E+17</v>
+      <c r="M77">
+        <v>0</v>
       </c>
       <c r="N77">
         <v>0</v>
@@ -4356,13 +4403,13 @@
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B78" t="s">
-        <v>176</v>
+        <v>105</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>106</v>
       </c>
       <c r="C78">
-        <v>126.58</v>
+        <v>136.23400000000001</v>
       </c>
       <c r="D78" s="4">
         <v>0</v>
@@ -4373,14 +4420,14 @@
       <c r="F78">
         <v>0</v>
       </c>
-      <c r="G78" s="12">
+      <c r="G78" s="13">
         <v>0</v>
       </c>
       <c r="H78">
         <v>0</v>
       </c>
-      <c r="I78" s="12">
-        <v>0</v>
+      <c r="I78" s="13">
+        <v>3.2841650965559202E+19</v>
       </c>
       <c r="J78">
         <v>0</v>
@@ -4391,22 +4438,22 @@
       <c r="L78">
         <v>0</v>
       </c>
-      <c r="M78" s="12">
-        <v>1.7506131971085699E+17</v>
+      <c r="M78">
+        <v>0</v>
       </c>
       <c r="N78">
         <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A79" s="3" t="s">
-        <v>177</v>
+      <c r="A79" t="s">
+        <v>107</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C79">
-        <v>161.03</v>
+        <v>170.24870000000001</v>
       </c>
       <c r="D79" s="4">
         <v>0</v>
@@ -4417,14 +4464,14 @@
       <c r="F79">
         <v>0</v>
       </c>
-      <c r="G79" s="12">
+      <c r="G79" s="13">
         <v>0</v>
       </c>
       <c r="H79">
-        <v>0</v>
-      </c>
-      <c r="I79" s="12">
-        <v>0</v>
+        <v>1375569322343650</v>
+      </c>
+      <c r="I79" s="13">
+        <v>5.9956572873684198E+17</v>
       </c>
       <c r="J79">
         <v>0</v>
@@ -4435,184 +4482,584 @@
       <c r="L79">
         <v>0</v>
       </c>
-      <c r="M79" s="12">
-        <v>6.98019330915034E+16</v>
-      </c>
-      <c r="N79">
-        <v>0</v>
+      <c r="M79">
+        <v>0</v>
+      </c>
+      <c r="N79" s="13">
+        <v>2.48918362198186E+16</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
+        <v>108</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C80">
+        <v>170.24870000000001</v>
+      </c>
+      <c r="D80" s="4">
+        <v>0</v>
+      </c>
+      <c r="E80">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>0</v>
+      </c>
+      <c r="G80" s="13">
+        <v>0</v>
+      </c>
+      <c r="H80">
+        <v>0</v>
+      </c>
+      <c r="I80" s="13">
+        <v>4.4569487799906803E+17</v>
+      </c>
+      <c r="J80">
+        <v>0</v>
+      </c>
+      <c r="K80">
+        <v>0</v>
+      </c>
+      <c r="L80">
+        <v>0</v>
+      </c>
+      <c r="M80">
+        <v>0</v>
+      </c>
+      <c r="N80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C81">
+        <v>204.3511</v>
+      </c>
+      <c r="D81" s="4">
+        <v>0</v>
+      </c>
+      <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>0</v>
+      </c>
+      <c r="G81" s="13">
+        <v>0</v>
+      </c>
+      <c r="H81">
+        <v>0</v>
+      </c>
+      <c r="I81" s="13">
+        <v>5.59185249900783E+18</v>
+      </c>
+      <c r="J81">
+        <v>0</v>
+      </c>
+      <c r="K81">
+        <v>0</v>
+      </c>
+      <c r="L81">
+        <v>0</v>
+      </c>
+      <c r="M81">
+        <v>0</v>
+      </c>
+      <c r="N81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A82" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B82" t="s">
+        <v>162</v>
+      </c>
+      <c r="C82">
+        <v>57.09</v>
+      </c>
+      <c r="D82" s="4">
+        <v>0</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>0</v>
+      </c>
+      <c r="G82" s="13">
+        <v>0</v>
+      </c>
+      <c r="H82">
+        <v>0</v>
+      </c>
+      <c r="I82" s="13">
+        <v>0</v>
+      </c>
+      <c r="J82">
+        <v>0</v>
+      </c>
+      <c r="K82">
+        <v>0</v>
+      </c>
+      <c r="L82">
+        <v>0</v>
+      </c>
+      <c r="M82" s="6">
+        <v>5062775445863580</v>
+      </c>
+      <c r="N82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A83" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B83" t="s">
+        <v>163</v>
+      </c>
+      <c r="C83">
+        <v>76.52</v>
+      </c>
+      <c r="D83" s="4">
+        <v>0</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>0</v>
+      </c>
+      <c r="G83" s="13">
+        <v>0</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83" s="13">
+        <v>0</v>
+      </c>
+      <c r="J83">
+        <v>0</v>
+      </c>
+      <c r="K83">
+        <v>0</v>
+      </c>
+      <c r="L83">
+        <v>0</v>
+      </c>
+      <c r="M83" s="14">
+        <v>2.0145241345485402E+17</v>
+      </c>
+      <c r="N83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A84" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C84">
+        <v>92.52</v>
+      </c>
+      <c r="D84" s="4">
+        <v>0</v>
+      </c>
+      <c r="E84">
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>0</v>
+      </c>
+      <c r="G84" s="13">
+        <v>0</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+      <c r="I84" s="13">
+        <v>0</v>
+      </c>
+      <c r="J84">
+        <v>0</v>
+      </c>
+      <c r="K84">
+        <v>0</v>
+      </c>
+      <c r="L84">
+        <v>0</v>
+      </c>
+      <c r="M84" s="14">
+        <v>8.43483998650832E+16</v>
+      </c>
+      <c r="N84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>165</v>
+      </c>
+      <c r="B85" t="s">
+        <v>166</v>
+      </c>
+      <c r="C85">
+        <v>123.1293</v>
+      </c>
+      <c r="D85" s="4">
+        <v>0</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="G85" s="13">
+        <v>0</v>
+      </c>
+      <c r="H85">
+        <v>0</v>
+      </c>
+      <c r="I85" s="13">
+        <v>0</v>
+      </c>
+      <c r="J85">
+        <v>0</v>
+      </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+      <c r="L85">
+        <v>0</v>
+      </c>
+      <c r="M85" s="14">
+        <v>1.09545383128709E+19</v>
+      </c>
+      <c r="N85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A86" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C86">
+        <v>106.1219</v>
+      </c>
+      <c r="D86" s="4">
+        <v>0</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>0</v>
+      </c>
+      <c r="G86" s="13">
+        <v>0</v>
+      </c>
+      <c r="H86">
+        <v>0</v>
+      </c>
+      <c r="I86" s="13">
+        <v>0</v>
+      </c>
+      <c r="J86">
+        <v>0</v>
+      </c>
+      <c r="K86">
+        <v>0</v>
+      </c>
+      <c r="L86">
+        <v>0</v>
+      </c>
+      <c r="M86" s="14">
+        <v>1.8157348621685801E+18</v>
+      </c>
+      <c r="N86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B87" t="s">
+        <v>170</v>
+      </c>
+      <c r="C87">
+        <v>107.15</v>
+      </c>
+      <c r="D87" s="4">
+        <v>0</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>0</v>
+      </c>
+      <c r="G87" s="13">
+        <v>0</v>
+      </c>
+      <c r="H87">
+        <v>0</v>
+      </c>
+      <c r="I87" s="13">
+        <v>0</v>
+      </c>
+      <c r="J87">
+        <v>0</v>
+      </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+      <c r="L87">
+        <v>0</v>
+      </c>
+      <c r="M87" s="14">
+        <v>6.8335892411046E+16</v>
+      </c>
+      <c r="N87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A88" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B88" t="s">
+        <v>172</v>
+      </c>
+      <c r="C88">
+        <v>126.58</v>
+      </c>
+      <c r="D88" s="4">
+        <v>0</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+      <c r="F88">
+        <v>0</v>
+      </c>
+      <c r="G88" s="13">
+        <v>0</v>
+      </c>
+      <c r="H88">
+        <v>0</v>
+      </c>
+      <c r="I88" s="13">
+        <v>0</v>
+      </c>
+      <c r="J88">
+        <v>0</v>
+      </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
+      <c r="L88">
+        <v>0</v>
+      </c>
+      <c r="M88" s="14">
+        <v>5.25183959132572E+16</v>
+      </c>
+      <c r="N88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A89" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C89">
+        <v>161.03</v>
+      </c>
+      <c r="D89" s="4">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>0</v>
+      </c>
+      <c r="F89">
+        <v>0</v>
+      </c>
+      <c r="G89" s="13">
+        <v>0</v>
+      </c>
+      <c r="H89">
+        <v>0</v>
+      </c>
+      <c r="I89" s="13">
+        <v>0</v>
+      </c>
+      <c r="J89">
+        <v>0</v>
+      </c>
+      <c r="K89">
+        <v>0</v>
+      </c>
+      <c r="L89">
+        <v>0</v>
+      </c>
+      <c r="M89" s="14">
+        <v>2.0940579927451E+16</v>
+      </c>
+      <c r="N89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>178</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C90">
+        <v>156.26</v>
+      </c>
+      <c r="D90" s="4">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>0</v>
+      </c>
+      <c r="F90">
+        <v>0</v>
+      </c>
+      <c r="G90" s="13">
+        <v>0</v>
+      </c>
+      <c r="H90">
+        <v>0</v>
+      </c>
+      <c r="I90" s="13">
+        <v>0</v>
+      </c>
+      <c r="J90">
+        <v>0</v>
+      </c>
+      <c r="K90">
+        <v>0</v>
+      </c>
+      <c r="L90">
+        <v>0</v>
+      </c>
+      <c r="M90" s="13">
+        <v>0</v>
+      </c>
+      <c r="N90" s="13">
+        <v>1.1865088354049E+16</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>181</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C91">
+        <v>158.28110000000001</v>
+      </c>
+      <c r="D91" s="4">
+        <v>0</v>
+      </c>
+      <c r="E91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <v>0</v>
+      </c>
+      <c r="G91" s="13">
+        <v>0</v>
+      </c>
+      <c r="H91">
+        <v>0</v>
+      </c>
+      <c r="I91" s="13">
+        <v>0</v>
+      </c>
+      <c r="J91">
+        <v>0</v>
+      </c>
+      <c r="K91">
+        <v>0</v>
+      </c>
+      <c r="L91">
+        <v>0</v>
+      </c>
+      <c r="M91" s="13">
+        <v>0</v>
+      </c>
+      <c r="N91">
+        <v>3831134091148240</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
         <v>183</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B92" t="s">
         <v>184</v>
       </c>
-      <c r="C80">
-        <v>156.26</v>
-      </c>
-      <c r="D80" s="4">
-        <v>0</v>
-      </c>
-      <c r="E80">
-        <v>0</v>
-      </c>
-      <c r="F80">
-        <v>0</v>
-      </c>
-      <c r="G80" s="12">
-        <v>0</v>
-      </c>
-      <c r="H80">
-        <v>0</v>
-      </c>
-      <c r="I80" s="12">
-        <v>0</v>
-      </c>
-      <c r="J80">
-        <v>0</v>
-      </c>
-      <c r="K80">
-        <v>0</v>
-      </c>
-      <c r="L80">
-        <v>0</v>
-      </c>
-      <c r="M80" s="12">
-        <v>0</v>
-      </c>
-      <c r="N80" s="12">
-        <v>1.1865088354049E+16</v>
-      </c>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>186</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="C81">
-        <v>158.28110000000001</v>
-      </c>
-      <c r="D81" s="4">
-        <v>0</v>
-      </c>
-      <c r="E81">
-        <v>0</v>
-      </c>
-      <c r="F81">
-        <v>0</v>
-      </c>
-      <c r="G81" s="12">
-        <v>0</v>
-      </c>
-      <c r="H81">
-        <v>0</v>
-      </c>
-      <c r="I81" s="12">
-        <v>0</v>
-      </c>
-      <c r="J81">
-        <v>0</v>
-      </c>
-      <c r="K81">
-        <v>0</v>
-      </c>
-      <c r="L81">
-        <v>0</v>
-      </c>
-      <c r="M81" s="12">
-        <v>0</v>
-      </c>
-      <c r="N81">
-        <v>3831134091148240</v>
-      </c>
-    </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>188</v>
-      </c>
-      <c r="B82" t="s">
-        <v>189</v>
-      </c>
-      <c r="C82">
+      <c r="C92">
         <v>122.12130000000001</v>
       </c>
-      <c r="D82" s="4">
-        <v>0</v>
-      </c>
-      <c r="E82">
-        <v>0</v>
-      </c>
-      <c r="F82">
-        <v>0</v>
-      </c>
-      <c r="G82" s="12">
-        <v>0</v>
-      </c>
-      <c r="H82">
-        <v>0</v>
-      </c>
-      <c r="I82" s="12">
-        <v>0</v>
-      </c>
-      <c r="J82">
-        <v>0</v>
-      </c>
-      <c r="K82">
-        <v>0</v>
-      </c>
-      <c r="L82">
-        <v>0</v>
-      </c>
-      <c r="M82" s="12">
-        <v>0</v>
-      </c>
-      <c r="N82" s="12">
+      <c r="D92" s="4">
+        <v>0</v>
+      </c>
+      <c r="E92">
+        <v>0</v>
+      </c>
+      <c r="F92">
+        <v>0</v>
+      </c>
+      <c r="G92" s="13">
+        <v>0</v>
+      </c>
+      <c r="H92">
+        <v>0</v>
+      </c>
+      <c r="I92" s="13">
+        <v>0</v>
+      </c>
+      <c r="J92">
+        <v>0</v>
+      </c>
+      <c r="K92">
+        <v>0</v>
+      </c>
+      <c r="L92">
+        <v>0</v>
+      </c>
+      <c r="M92" s="13">
+        <v>0</v>
+      </c>
+      <c r="N92" s="13">
         <v>1.82639924706312E+16</v>
       </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A83" s="3"/>
-      <c r="B83" s="3"/>
-    </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A84" s="3"/>
-      <c r="B84" s="3"/>
-    </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A85" s="3"/>
-      <c r="B85" s="3"/>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A86" s="3"/>
-      <c r="B86" s="3"/>
-    </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A87" s="3"/>
-      <c r="B87" s="3"/>
-    </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A88" s="3"/>
-      <c r="B88" s="3"/>
-    </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A89" s="3"/>
-      <c r="B89" s="3"/>
-    </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A90" s="3"/>
-      <c r="B90" s="3"/>
-    </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A91" s="3"/>
-      <c r="B91" s="3"/>
-    </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A92" s="3"/>
-      <c r="B92" s="3"/>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A93" s="3"/>
@@ -44674,9 +45121,49 @@
       <c r="A10107" s="3"/>
       <c r="B10107" s="3"/>
     </row>
-    <row r="10108" spans="1:2" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10108" s="5"/>
+    <row r="10108" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10108" s="3"/>
       <c r="B10108" s="3"/>
+    </row>
+    <row r="10109" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10109" s="3"/>
+      <c r="B10109" s="3"/>
+    </row>
+    <row r="10110" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10110" s="3"/>
+      <c r="B10110" s="3"/>
+    </row>
+    <row r="10111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10111" s="3"/>
+      <c r="B10111" s="3"/>
+    </row>
+    <row r="10112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10112" s="3"/>
+      <c r="B10112" s="3"/>
+    </row>
+    <row r="10113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10113" s="3"/>
+      <c r="B10113" s="3"/>
+    </row>
+    <row r="10114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10114" s="3"/>
+      <c r="B10114" s="3"/>
+    </row>
+    <row r="10115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10115" s="3"/>
+      <c r="B10115" s="3"/>
+    </row>
+    <row r="10116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10116" s="3"/>
+      <c r="B10116" s="3"/>
+    </row>
+    <row r="10117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10117" s="3"/>
+      <c r="B10117" s="3"/>
+    </row>
+    <row r="10118" spans="1:2" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10118" s="5"/>
+      <c r="B10118" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -44697,15 +45184,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="32" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B1" t="s">
-        <v>164</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -44722,6 +45209,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6030F4CF-2F4B-594A-AF9C-1A8D5AE0E84E}">
   <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.5" customWidth="1"/>
+    <col min="9" max="9" width="28.5" customWidth="1"/>
+    <col min="10" max="10" width="20.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -45066,27 +45558,27 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated indoor_environment_PyCHAM_setup to be user-friendly
now much clearer which variables to change to prepare sensitivity simulations
</commit_message>
<xml_diff>
--- a/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
+++ b/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Documents/GitHub/NCAS-BoxModellingToolkit/indoor_environment_PyCHAM_setup/src/indoor_environment_PyCHAM_setup/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livemanchesterac-my.sharepoint.com/personal/simon_omeara_manchester_ac_uk/Documents/GitHub/NCAS-BoxModellingToolkit/indoor_environment_PyCHAM_setup/src/indoor_environment_PyCHAM_setup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63E5A6B-FED0-9348-BDAA-8DBBD09655F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{2EF619C7-E479-174A-A447-3F7B7DC38047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5673C54A-211E-594B-B3B8-AA074746E0F4}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="5900" windowWidth="31060" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2460" yWindow="500" windowWidth="21860" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_emi" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="202">
   <si>
     <t>ACRYLONITRILE</t>
   </si>
@@ -605,9 +605,6 @@
     <t>in Table 1 they give the mass fraction of PM10 that is PM2.5 and they give the number of PM10  particles emitted/min emission rate, whilst their Figure  3 indicates that particle number concentration for washable filter bag less vacuum is dominated by PM2.5 (with a mean radius around 0.015 um), which is consistent with Figure 14 of doi.org/10.1016/j.atmosenv.2010.01.009. To get emission rate of PM2.5 particles in number/unit of time, first multiply the mass emission rate of PM10 (ug/s) from their Table 1 by 0.742 (the mass fraction that is PM2.5 from their Table 1), giving 0.93492 ug/s, then get mass of one particle of radius 0.015 um (radius set for vacuum cleaning for PM2.5 in indoor_emi sheet of this file), assuming a density of 1.4e-6 ug/um3, giving (using mass emission rate of PM10 (ug/s) from the washable filter bag less vacuum in their Table 1): (0.742*1.26)/((4./3.)*np.pi*0.015**3*1.4e-6) = 4.7e10 particles/s of PM2.5 with a mean radius of 0.015 um, likewise, the same can be done for PM2.5-PM10 assuming a mean radius of 2.5 um: ((1.-0.742)*1.26)/((4./3.)*np.pi*2.5**3*1.4e-6) = 3.5e3 particles/s of PM2.5-PM10 with a mean radius of 2.5 um</t>
   </si>
   <si>
-    <t>Frying (these values represent particles/ or molecules/s/person/meal or mole fraction of particles; particles from 10.1016/j.atmosenv.2010.01.009, using Table 2, which gives units in /min, and so /60 to convert to /s, e.g. 8.02e12 particles/60, gases from https://onlinelibrary.wiley.com/doi/full/10.1111/ina.12906 (Table 4), assuming stir fry lasted 15 minutes, e.g. for ethanol from table 4: ((67.e-3/46.0684)*6.022e23)/(15.*60.), note that citral not in MCM, so represented by limonene).  Particle radius of 0.03 um is suggested by Figure 12 of this reference. Black carbon to primary organic mole fractions estimated from Table 18 of http://dx.doi.org/10.1016/j.atmosenv.2013.01.061</t>
-  </si>
-  <si>
     <t>page 660 of https://doi.org/10.1080/15459624.2019.1643466 says the mass fraction of cleaning spray emitted on a single spray that goes airbourne (as gas and particles) rather than deposit on the surface to be cleaned is up to 1/3 (backed up by Figure S5 of https://doi.org/10.1016/j.ijheh.2023.114220), also mass of airbourne particles from cleaning spray is small (maximum mass fraction compared to airbourne particles+gas is 0.01%) compared to gas-phase from cleaning spray. Article https://doi.org/10.1016/j.ijheh.2023.114220 says the average emission rate (of total material (airbourne+deposited) is 1.6 g/s of cleaning spray). Suggest the following: convert the size-resolved plots of particle in the paper (Fig. 3 which suggests that the ratio in PM2.5 to PM10 is about 50:50) into an emission rate of particle containing a non-volatile material, and convert the mass of VOC released into individual components based on a mass-weighted ingredient list. This website (https://www.statista.com/statistics/304000/leading-brands-of-household-cleaners-in-the-uk/) suggests Dettol anti-bacterial surface cleanser is one of the best selling in the UK. The back of the dettol bottle lists: benzalkonium chloride as 0.096 % by mass, then there is also an unamed fragrance, sodium bicarbonate, sodium carbonate, sodium edetate, water, C9-C11 alkylpolyglycoside and C12-C16 Pareth-7. I think I can use this article (https://doi.org/10.1039/D2EA00054G) to get the VOC emission rates for commercial cleaning products, and the same article indicates that benzalkonium chloride is non-volatile (which the girolami techqnique estimates to have a density of 0.86g/cm^3), so this along with the sodium salts could represent the non-volatile particles</t>
   </si>
   <si>
@@ -643,6 +640,12 @@
   <si>
     <t>mean_rad_pm2</t>
   </si>
+  <si>
+    <t>this paper 10.1021/es202946w (emission rates of PM2.5 (ug/min) in Table 1 gives similar values to those reported in https://doi.org/10.1016/j.buildenv.2020.107059, though notes that in certan tests the emission rate was up to 3 orders of magnitude higher), it is noted that https://doi.org/10.1016/j.buildenv.2020.107059 does not account for particle loss to indoor surfaces, therefore values were increased by a factor 2.5 to correct for this</t>
+  </si>
+  <si>
+    <t>Frying (these values represent particles/ or molecules/s/person/meal or mole fraction of particles; particles from 10.1016/j.atmosenv.2010.01.009, using Table 2, which gives units in /min, and so /60 to convert to /s, e.g. 8.02e12 particles/60, gases from https://onlinelibrary.wiley.com/doi/full/10.1111/ina.12906 (Table 4), assuming stir fry lasted 15 minutes, e.g. for ethanol from table 4: ((67.e-3/46.0684)*6.022e23)/(15.*60.), note that citral not in MCM, so represented by limonene).  Particle radius of 0.03 um is suggested by Figure 12 of this reference (10.1016/j.atmosenv.2010.01.009). Black carbon to primary organic mole fractions estimated from Table 18 of http://dx.doi.org/10.1016/j.atmosenv.2013.01.061</t>
+  </si>
 </sst>
 </file>
 
@@ -673,8 +676,9 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Menlo"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -727,7 +731,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
@@ -747,6 +750,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1042,7 +1046,7 @@
     <col min="5" max="5" width="32.1640625" customWidth="1"/>
     <col min="6" max="6" width="22.33203125" customWidth="1"/>
     <col min="7" max="7" width="19.5" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
     <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.83203125" bestFit="1" customWidth="1"/>
@@ -1052,9 +1056,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="7"/>
-      <c r="B1" s="7"/>
-      <c r="C1" s="8"/>
+      <c r="A1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="7"/>
       <c r="D1" s="15" t="s">
         <v>161</v>
       </c>
@@ -1062,103 +1066,103 @@
       <c r="F1" s="15"/>
       <c r="G1" s="15"/>
       <c r="H1" s="15"/>
-      <c r="I1" s="9"/>
+      <c r="I1" s="8"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="F2" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="G2" s="9" t="s">
+      <c r="F2" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="L2" s="9" t="s">
+      <c r="L2" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="M2" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="N2" s="9" t="s">
+      <c r="M2" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="N2" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="8" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="11">
-        <v>0</v>
-      </c>
-      <c r="D3" s="11">
+      <c r="C3" s="10">
+        <v>0</v>
+      </c>
+      <c r="D3" s="10">
         <v>0</v>
       </c>
       <c r="E3">
         <v>147166666666.67001</v>
       </c>
-      <c r="F3">
-        <v>133666666666.7</v>
-      </c>
-      <c r="G3" s="9">
-        <v>0</v>
-      </c>
-      <c r="H3" s="9">
-        <v>0</v>
-      </c>
-      <c r="I3" s="9">
-        <v>0</v>
-      </c>
-      <c r="J3" s="9">
+      <c r="F3" s="13">
+        <v>395510416666.67499</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3" s="8">
+        <v>0</v>
+      </c>
+      <c r="I3" s="8">
+        <v>0</v>
+      </c>
+      <c r="J3" s="8">
         <v>1317449251.0999999</v>
       </c>
-      <c r="K3" s="9">
-        <v>0</v>
-      </c>
-      <c r="L3" s="13">
-        <v>47000000000</v>
-      </c>
-      <c r="M3" s="6">
-        <v>0</v>
-      </c>
-      <c r="N3" s="9">
-        <v>0</v>
-      </c>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
+      <c r="K3" s="8">
+        <v>0</v>
+      </c>
+      <c r="L3" s="12">
+        <v>117500000000</v>
+      </c>
+      <c r="M3" s="13">
+        <v>0</v>
+      </c>
+      <c r="N3" s="8">
+        <v>0</v>
+      </c>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
@@ -1203,8 +1207,8 @@
       <c r="N4">
         <v>0</v>
       </c>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
@@ -1249,8 +1253,8 @@
       <c r="N5">
         <v>0</v>
       </c>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
@@ -1295,8 +1299,8 @@
       <c r="N6">
         <v>0</v>
       </c>
-      <c r="O6" s="9"/>
-      <c r="P6" s="9"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
@@ -1341,8 +1345,8 @@
       <c r="N7">
         <v>0</v>
       </c>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
@@ -1385,8 +1389,8 @@
       <c r="N8">
         <v>0</v>
       </c>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
@@ -1429,8 +1433,8 @@
       <c r="N9">
         <v>0</v>
       </c>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
@@ -1473,8 +1477,8 @@
       <c r="N10">
         <v>0</v>
       </c>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
@@ -1517,8 +1521,8 @@
       <c r="N11">
         <v>0</v>
       </c>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
@@ -1534,7 +1538,7 @@
         <v>3.9E-2</v>
       </c>
       <c r="F12">
-        <v>0.03</v>
+        <v>2.4E-2</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1560,20 +1564,20 @@
       <c r="N12">
         <v>0</v>
       </c>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>52</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C13" s="11">
-        <v>0</v>
-      </c>
-      <c r="D13" s="11">
+      <c r="C13" s="10">
+        <v>0</v>
+      </c>
+      <c r="D13" s="10">
         <v>0</v>
       </c>
       <c r="E13">
@@ -1582,28 +1586,28 @@
       <c r="F13">
         <v>0</v>
       </c>
-      <c r="G13" s="9">
-        <v>0</v>
-      </c>
-      <c r="H13" s="9">
-        <v>0</v>
-      </c>
-      <c r="I13" s="9">
-        <v>0</v>
-      </c>
-      <c r="J13" s="9">
-        <v>0</v>
-      </c>
-      <c r="K13" s="9">
-        <v>0</v>
-      </c>
-      <c r="L13" s="13">
-        <v>0</v>
-      </c>
-      <c r="M13" s="6">
+      <c r="G13" s="8">
+        <v>0</v>
+      </c>
+      <c r="H13" s="8">
+        <v>0</v>
+      </c>
+      <c r="I13" s="8">
+        <v>0</v>
+      </c>
+      <c r="J13" s="8">
+        <v>0</v>
+      </c>
+      <c r="K13" s="8">
+        <v>0</v>
+      </c>
+      <c r="L13" s="12">
+        <v>0</v>
+      </c>
+      <c r="M13" s="13">
         <v>2220766.6477938802</v>
       </c>
-      <c r="N13" s="9">
+      <c r="N13" s="8">
         <v>0</v>
       </c>
     </row>
@@ -1993,8 +1997,8 @@
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
-        <v>191</v>
+      <c r="A23" s="11" t="s">
+        <v>190</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>146</v>
@@ -2026,10 +2030,10 @@
       <c r="K23">
         <v>0</v>
       </c>
-      <c r="L23" s="13">
-        <v>3500</v>
-      </c>
-      <c r="M23" s="6">
+      <c r="L23" s="12">
+        <v>8750</v>
+      </c>
+      <c r="M23" s="13">
         <v>142129.06545880801</v>
       </c>
       <c r="N23">
@@ -2037,8 +2041,8 @@
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A24" s="12" t="s">
-        <v>192</v>
+      <c r="A24" s="11" t="s">
+        <v>191</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>145</v>
@@ -2082,7 +2086,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>150</v>
@@ -2126,7 +2130,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>148</v>
@@ -2170,7 +2174,7 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>158</v>
@@ -2214,7 +2218,7 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28">
@@ -2256,7 +2260,7 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29">
@@ -2298,7 +2302,7 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30">
@@ -2340,7 +2344,7 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31">
@@ -2382,7 +2386,7 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>147</v>
@@ -2490,7 +2494,7 @@
       <c r="H34">
         <v>0</v>
       </c>
-      <c r="I34" s="13">
+      <c r="I34" s="12">
         <v>7.4580997301490002E+18</v>
       </c>
       <c r="J34">
@@ -2569,7 +2573,7 @@
       <c r="E36">
         <v>0</v>
       </c>
-      <c r="F36" s="13">
+      <c r="F36" s="12">
         <v>9.7312788037883699E+17</v>
       </c>
       <c r="G36">
@@ -2578,7 +2582,7 @@
       <c r="H36">
         <v>0</v>
       </c>
-      <c r="I36" s="13">
+      <c r="I36" s="12">
         <v>5.8707519291711396E+21</v>
       </c>
       <c r="J36">
@@ -2613,10 +2617,10 @@
       <c r="E37">
         <v>0</v>
       </c>
-      <c r="F37" s="13">
+      <c r="F37" s="12">
         <v>8.9794231234033504E+16</v>
       </c>
-      <c r="G37" s="13">
+      <c r="G37" s="12">
         <v>2.2135322118157E+16</v>
       </c>
       <c r="H37">
@@ -2657,7 +2661,7 @@
       <c r="E38">
         <v>0</v>
       </c>
-      <c r="F38" s="13">
+      <c r="F38" s="12">
         <v>3.89976834891242E+16</v>
       </c>
       <c r="G38">
@@ -2666,7 +2670,7 @@
       <c r="H38">
         <v>0</v>
       </c>
-      <c r="I38" s="13">
+      <c r="I38" s="12">
         <v>0</v>
       </c>
       <c r="J38">
@@ -2701,16 +2705,16 @@
       <c r="E39">
         <v>0</v>
       </c>
-      <c r="F39" s="13">
+      <c r="F39" s="12">
         <v>2.56692630577486E+16</v>
       </c>
-      <c r="G39" s="13">
+      <c r="G39" s="12">
         <v>1.57964695739991E+16</v>
       </c>
       <c r="H39">
         <v>0</v>
       </c>
-      <c r="I39" s="13">
+      <c r="I39" s="12">
         <v>1.7593729219433099E+19</v>
       </c>
       <c r="J39">
@@ -2745,7 +2749,7 @@
       <c r="E40">
         <v>0</v>
       </c>
-      <c r="F40" s="13">
+      <c r="F40" s="12">
         <v>1.47464788921009E+16</v>
       </c>
       <c r="G40">
@@ -2754,7 +2758,7 @@
       <c r="H40">
         <v>0</v>
       </c>
-      <c r="I40" s="13">
+      <c r="I40" s="12">
         <v>1.88E+19</v>
       </c>
       <c r="J40">
@@ -2798,7 +2802,7 @@
       <c r="H41">
         <v>0</v>
       </c>
-      <c r="I41" s="13">
+      <c r="I41" s="12">
         <v>0</v>
       </c>
       <c r="J41">
@@ -2830,19 +2834,19 @@
       <c r="D42" s="4">
         <v>0</v>
       </c>
-      <c r="E42" s="13">
+      <c r="E42" s="12">
         <v>6494526650446900</v>
       </c>
-      <c r="F42" s="13">
-        <v>0</v>
-      </c>
-      <c r="G42" s="13">
+      <c r="F42" s="12">
+        <v>0</v>
+      </c>
+      <c r="G42" s="12">
         <v>0</v>
       </c>
       <c r="H42">
         <v>0</v>
       </c>
-      <c r="I42" s="13">
+      <c r="I42" s="12">
         <v>0</v>
       </c>
       <c r="J42">
@@ -2874,19 +2878,19 @@
       <c r="D43" s="4">
         <v>0</v>
       </c>
-      <c r="E43" s="13">
+      <c r="E43" s="12">
         <v>4.05206901116216E+16</v>
       </c>
       <c r="F43">
         <v>3438038799255520</v>
       </c>
-      <c r="G43" s="13">
+      <c r="G43" s="12">
         <v>0</v>
       </c>
       <c r="H43">
         <v>0</v>
       </c>
-      <c r="I43" s="13">
+      <c r="I43" s="12">
         <v>2.7450925701073101E+18</v>
       </c>
       <c r="J43">
@@ -2924,13 +2928,13 @@
       <c r="F44">
         <v>6683556305501490</v>
       </c>
-      <c r="G44" s="13">
+      <c r="G44" s="12">
         <v>0</v>
       </c>
       <c r="H44">
         <v>0</v>
       </c>
-      <c r="I44" s="13">
+      <c r="I44" s="12">
         <v>0</v>
       </c>
       <c r="J44">
@@ -2968,13 +2972,13 @@
       <c r="F45">
         <v>0</v>
       </c>
-      <c r="G45" s="13">
+      <c r="G45" s="12">
         <v>0</v>
       </c>
       <c r="H45">
         <v>0</v>
       </c>
-      <c r="I45" s="13">
+      <c r="I45" s="12">
         <v>0</v>
       </c>
       <c r="J45">
@@ -3009,16 +3013,16 @@
       <c r="E46">
         <v>3855758491862170</v>
       </c>
-      <c r="F46" s="13">
-        <v>0</v>
-      </c>
-      <c r="G46" s="13">
+      <c r="F46" s="12">
+        <v>0</v>
+      </c>
+      <c r="G46" s="12">
         <v>0</v>
       </c>
       <c r="H46">
         <v>0</v>
       </c>
-      <c r="I46" s="13">
+      <c r="I46" s="12">
         <v>0</v>
       </c>
       <c r="J46">
@@ -3050,19 +3054,19 @@
       <c r="D47" s="4">
         <v>0</v>
       </c>
-      <c r="E47" s="13">
+      <c r="E47" s="12">
         <v>2.30306213752953E+16</v>
       </c>
       <c r="F47">
         <v>0</v>
       </c>
-      <c r="G47" s="13">
+      <c r="G47" s="12">
         <v>0</v>
       </c>
       <c r="H47">
         <v>0</v>
       </c>
-      <c r="I47" s="13">
+      <c r="I47" s="12">
         <v>0</v>
       </c>
       <c r="J47">
@@ -3097,16 +3101,16 @@
       <c r="E48">
         <v>4972719602159980</v>
       </c>
-      <c r="F48" s="13">
-        <v>0</v>
-      </c>
-      <c r="G48" s="13">
+      <c r="F48" s="12">
+        <v>0</v>
+      </c>
+      <c r="G48" s="12">
         <v>0</v>
       </c>
       <c r="H48">
         <v>0</v>
       </c>
-      <c r="I48" s="13">
+      <c r="I48" s="12">
         <v>2.8332937268120801E+18</v>
       </c>
       <c r="J48">
@@ -3144,7 +3148,7 @@
       <c r="F49">
         <v>0</v>
       </c>
-      <c r="G49" s="13">
+      <c r="G49" s="12">
         <v>0</v>
       </c>
       <c r="H49">
@@ -3185,16 +3189,16 @@
       <c r="E50">
         <v>1181757319581150</v>
       </c>
-      <c r="F50" s="13">
-        <v>0</v>
-      </c>
-      <c r="G50" s="13">
+      <c r="F50" s="12">
+        <v>0</v>
+      </c>
+      <c r="G50" s="12">
         <v>0</v>
       </c>
       <c r="H50">
         <v>0</v>
       </c>
-      <c r="I50" s="13">
+      <c r="I50" s="12">
         <v>0</v>
       </c>
       <c r="J50">
@@ -3232,13 +3236,13 @@
       <c r="F51">
         <v>0</v>
       </c>
-      <c r="G51" s="13">
+      <c r="G51" s="12">
         <v>0</v>
       </c>
       <c r="H51">
         <v>0</v>
       </c>
-      <c r="I51" s="13">
+      <c r="I51" s="12">
         <v>0</v>
       </c>
       <c r="J51">
@@ -3273,16 +3277,16 @@
       <c r="E52">
         <v>671238157522096</v>
       </c>
-      <c r="F52" s="13">
-        <v>0</v>
-      </c>
-      <c r="G52" s="13">
+      <c r="F52" s="12">
+        <v>0</v>
+      </c>
+      <c r="G52" s="12">
         <v>0</v>
       </c>
       <c r="H52">
         <v>0</v>
       </c>
-      <c r="I52" s="13">
+      <c r="I52" s="12">
         <v>0</v>
       </c>
       <c r="J52">
@@ -3320,13 +3324,13 @@
       <c r="F53">
         <v>0</v>
       </c>
-      <c r="G53" s="13">
+      <c r="G53" s="12">
         <v>0</v>
       </c>
       <c r="H53">
         <v>0</v>
       </c>
-      <c r="I53" s="13">
+      <c r="I53" s="12">
         <v>0</v>
       </c>
       <c r="J53">
@@ -3361,16 +3365,16 @@
       <c r="E54">
         <v>459291306269878</v>
       </c>
-      <c r="F54" s="13">
-        <v>0</v>
-      </c>
-      <c r="G54" s="13">
+      <c r="F54" s="12">
+        <v>0</v>
+      </c>
+      <c r="G54" s="12">
         <v>0</v>
       </c>
       <c r="H54">
         <v>0</v>
       </c>
-      <c r="I54" s="13">
+      <c r="I54" s="12">
         <v>0</v>
       </c>
       <c r="J54">
@@ -3408,13 +3412,13 @@
       <c r="F55">
         <v>0</v>
       </c>
-      <c r="G55" s="13">
+      <c r="G55" s="12">
         <v>0</v>
       </c>
       <c r="H55">
         <v>0</v>
       </c>
-      <c r="I55" s="13">
+      <c r="I55" s="12">
         <v>0</v>
       </c>
       <c r="J55">
@@ -3449,16 +3453,16 @@
       <c r="E56">
         <v>115049465648389</v>
       </c>
-      <c r="F56" s="13">
-        <v>0</v>
-      </c>
-      <c r="G56" s="13">
+      <c r="F56" s="12">
+        <v>0</v>
+      </c>
+      <c r="G56" s="12">
         <v>0</v>
       </c>
       <c r="H56">
         <v>0</v>
       </c>
-      <c r="I56" s="13">
+      <c r="I56" s="12">
         <v>0</v>
       </c>
       <c r="J56">
@@ -3496,13 +3500,13 @@
       <c r="F57">
         <v>0</v>
       </c>
-      <c r="G57" s="13">
+      <c r="G57" s="12">
         <v>0</v>
       </c>
       <c r="H57">
         <v>0</v>
       </c>
-      <c r="I57" s="13">
+      <c r="I57" s="12">
         <v>0</v>
       </c>
       <c r="J57">
@@ -3537,16 +3541,16 @@
       <c r="E58">
         <v>885189865959984</v>
       </c>
-      <c r="F58" s="13">
-        <v>0</v>
-      </c>
-      <c r="G58" s="13">
+      <c r="F58" s="12">
+        <v>0</v>
+      </c>
+      <c r="G58" s="12">
         <v>0</v>
       </c>
       <c r="H58">
         <v>0</v>
       </c>
-      <c r="I58" s="13">
+      <c r="I58" s="12">
         <v>0</v>
       </c>
       <c r="J58">
@@ -3584,13 +3588,13 @@
       <c r="F59">
         <v>0</v>
       </c>
-      <c r="G59" s="13">
+      <c r="G59" s="12">
         <v>0</v>
       </c>
       <c r="H59">
         <v>0</v>
       </c>
-      <c r="I59" s="13">
+      <c r="I59" s="12">
         <v>0</v>
       </c>
       <c r="J59">
@@ -3625,16 +3629,16 @@
       <c r="E60">
         <v>213476443143224</v>
       </c>
-      <c r="F60" s="13">
-        <v>0</v>
-      </c>
-      <c r="G60" s="13">
+      <c r="F60" s="12">
+        <v>0</v>
+      </c>
+      <c r="G60" s="12">
         <v>0</v>
       </c>
       <c r="H60">
         <v>0</v>
       </c>
-      <c r="I60" s="13">
+      <c r="I60" s="12">
         <v>0</v>
       </c>
       <c r="J60">
@@ -3672,13 +3676,13 @@
       <c r="F61">
         <v>0</v>
       </c>
-      <c r="G61" s="13">
+      <c r="G61" s="12">
         <v>0</v>
       </c>
       <c r="H61">
         <v>0</v>
       </c>
-      <c r="I61" s="13">
+      <c r="I61" s="12">
         <v>0</v>
       </c>
       <c r="J61">
@@ -3713,16 +3717,16 @@
       <c r="E62">
         <v>1422603851820030</v>
       </c>
-      <c r="F62" s="13">
-        <v>0</v>
-      </c>
-      <c r="G62" s="13">
+      <c r="F62" s="12">
+        <v>0</v>
+      </c>
+      <c r="G62" s="12">
         <v>0</v>
       </c>
       <c r="H62">
         <v>0</v>
       </c>
-      <c r="I62" s="13">
+      <c r="I62" s="12">
         <v>0</v>
       </c>
       <c r="J62">
@@ -3760,13 +3764,13 @@
       <c r="F63">
         <v>0</v>
       </c>
-      <c r="G63" s="13">
+      <c r="G63" s="12">
         <v>0</v>
       </c>
       <c r="H63">
         <v>0</v>
       </c>
-      <c r="I63" s="13">
+      <c r="I63" s="12">
         <v>0</v>
       </c>
       <c r="J63">
@@ -3801,16 +3805,16 @@
       <c r="E64">
         <v>4144017962239770</v>
       </c>
-      <c r="F64" s="13">
-        <v>0</v>
-      </c>
-      <c r="G64" s="13">
+      <c r="F64" s="12">
+        <v>0</v>
+      </c>
+      <c r="G64" s="12">
         <v>0</v>
       </c>
       <c r="H64">
         <v>0</v>
       </c>
-      <c r="I64" s="13">
+      <c r="I64" s="12">
         <v>0</v>
       </c>
       <c r="J64">
@@ -3848,13 +3852,13 @@
       <c r="F65">
         <v>0</v>
       </c>
-      <c r="G65" s="13">
+      <c r="G65" s="12">
         <v>0</v>
       </c>
       <c r="H65">
         <v>0</v>
       </c>
-      <c r="I65" s="13">
+      <c r="I65" s="12">
         <v>0</v>
       </c>
       <c r="J65">
@@ -3889,16 +3893,16 @@
       <c r="E66">
         <v>9898568768132020</v>
       </c>
-      <c r="F66" s="13">
-        <v>0</v>
-      </c>
-      <c r="G66" s="13">
+      <c r="F66" s="12">
+        <v>0</v>
+      </c>
+      <c r="G66" s="12">
         <v>0</v>
       </c>
       <c r="H66">
         <v>0</v>
       </c>
-      <c r="I66" s="13">
+      <c r="I66" s="12">
         <v>0</v>
       </c>
       <c r="J66">
@@ -3936,13 +3940,13 @@
       <c r="F67">
         <v>0</v>
       </c>
-      <c r="G67" s="13">
+      <c r="G67" s="12">
         <v>0</v>
       </c>
       <c r="H67">
         <v>0</v>
       </c>
-      <c r="I67" s="13">
+      <c r="I67" s="12">
         <v>0</v>
       </c>
       <c r="J67">
@@ -3980,10 +3984,10 @@
       <c r="F68">
         <v>2996005239351240</v>
       </c>
-      <c r="G68" s="13">
-        <v>0</v>
-      </c>
-      <c r="H68" s="13">
+      <c r="G68" s="12">
+        <v>0</v>
+      </c>
+      <c r="H68" s="12">
         <v>6.13935499867058E+16</v>
       </c>
       <c r="I68">
@@ -4024,7 +4028,7 @@
       <c r="F69">
         <v>0</v>
       </c>
-      <c r="G69" s="13">
+      <c r="G69" s="12">
         <v>0</v>
       </c>
       <c r="H69">
@@ -4068,13 +4072,13 @@
       <c r="F70">
         <v>0</v>
       </c>
-      <c r="G70" s="13">
+      <c r="G70" s="12">
         <v>0</v>
       </c>
       <c r="H70">
         <v>0</v>
       </c>
-      <c r="I70" s="13">
+      <c r="I70" s="12">
         <v>0</v>
       </c>
       <c r="J70">
@@ -4112,16 +4116,16 @@
       <c r="F71">
         <v>0</v>
       </c>
-      <c r="G71" s="13">
+      <c r="G71" s="12">
         <v>0</v>
       </c>
       <c r="H71">
         <v>0</v>
       </c>
-      <c r="I71" s="13">
-        <v>0</v>
-      </c>
-      <c r="J71" s="13">
+      <c r="I71" s="12">
+        <v>0</v>
+      </c>
+      <c r="J71" s="12">
         <v>4.7866168828592902E+17</v>
       </c>
       <c r="K71">
@@ -4156,13 +4160,13 @@
       <c r="F72">
         <v>0</v>
       </c>
-      <c r="G72" s="13">
+      <c r="G72" s="12">
         <v>0</v>
       </c>
       <c r="H72">
         <v>0</v>
       </c>
-      <c r="I72" s="13">
+      <c r="I72" s="12">
         <v>0</v>
       </c>
       <c r="J72">
@@ -4200,13 +4204,13 @@
       <c r="F73">
         <v>0</v>
       </c>
-      <c r="G73" s="13">
+      <c r="G73" s="12">
         <v>0</v>
       </c>
       <c r="H73">
         <v>0</v>
       </c>
-      <c r="I73" s="13">
+      <c r="I73" s="12">
         <v>0</v>
       </c>
       <c r="J73">
@@ -4244,13 +4248,13 @@
       <c r="F74">
         <v>0</v>
       </c>
-      <c r="G74" s="13">
+      <c r="G74" s="12">
         <v>0</v>
       </c>
       <c r="H74">
         <v>0</v>
       </c>
-      <c r="I74" s="13">
+      <c r="I74" s="12">
         <v>7.99324851692944E+17</v>
       </c>
       <c r="J74">
@@ -4288,13 +4292,13 @@
       <c r="F75">
         <v>0</v>
       </c>
-      <c r="G75" s="13">
+      <c r="G75" s="12">
         <v>0</v>
       </c>
       <c r="H75">
         <v>0</v>
       </c>
-      <c r="I75" s="13">
+      <c r="I75" s="12">
         <v>2.8727962844572001E+18</v>
       </c>
       <c r="J75">
@@ -4332,13 +4336,13 @@
       <c r="F76">
         <v>0</v>
       </c>
-      <c r="G76" s="13">
+      <c r="G76" s="12">
         <v>0</v>
       </c>
       <c r="H76">
         <v>0</v>
       </c>
-      <c r="I76" s="13">
+      <c r="I76" s="12">
         <v>2.1374745930516401E+18</v>
       </c>
       <c r="J76">
@@ -4376,13 +4380,13 @@
       <c r="F77">
         <v>0</v>
       </c>
-      <c r="G77" s="13">
+      <c r="G77" s="12">
         <v>0</v>
       </c>
       <c r="H77">
         <v>0</v>
       </c>
-      <c r="I77" s="13">
+      <c r="I77" s="12">
         <v>7.0407870654329997E+17</v>
       </c>
       <c r="J77">
@@ -4420,13 +4424,13 @@
       <c r="F78">
         <v>0</v>
       </c>
-      <c r="G78" s="13">
+      <c r="G78" s="12">
         <v>0</v>
       </c>
       <c r="H78">
         <v>0</v>
       </c>
-      <c r="I78" s="13">
+      <c r="I78" s="12">
         <v>3.2841650965559202E+19</v>
       </c>
       <c r="J78">
@@ -4464,13 +4468,13 @@
       <c r="F79">
         <v>0</v>
       </c>
-      <c r="G79" s="13">
+      <c r="G79" s="12">
         <v>0</v>
       </c>
       <c r="H79">
         <v>1375569322343650</v>
       </c>
-      <c r="I79" s="13">
+      <c r="I79" s="12">
         <v>5.9956572873684198E+17</v>
       </c>
       <c r="J79">
@@ -4485,7 +4489,7 @@
       <c r="M79">
         <v>0</v>
       </c>
-      <c r="N79" s="13">
+      <c r="N79" s="12">
         <v>2.48918362198186E+16</v>
       </c>
     </row>
@@ -4508,13 +4512,13 @@
       <c r="F80">
         <v>0</v>
       </c>
-      <c r="G80" s="13">
+      <c r="G80" s="12">
         <v>0</v>
       </c>
       <c r="H80">
         <v>0</v>
       </c>
-      <c r="I80" s="13">
+      <c r="I80" s="12">
         <v>4.4569487799906803E+17</v>
       </c>
       <c r="J80">
@@ -4552,13 +4556,13 @@
       <c r="F81">
         <v>0</v>
       </c>
-      <c r="G81" s="13">
+      <c r="G81" s="12">
         <v>0</v>
       </c>
       <c r="H81">
         <v>0</v>
       </c>
-      <c r="I81" s="13">
+      <c r="I81" s="12">
         <v>5.59185249900783E+18</v>
       </c>
       <c r="J81">
@@ -4596,13 +4600,13 @@
       <c r="F82">
         <v>0</v>
       </c>
-      <c r="G82" s="13">
+      <c r="G82" s="12">
         <v>0</v>
       </c>
       <c r="H82">
         <v>0</v>
       </c>
-      <c r="I82" s="13">
+      <c r="I82" s="12">
         <v>0</v>
       </c>
       <c r="J82">
@@ -4614,7 +4618,7 @@
       <c r="L82">
         <v>0</v>
       </c>
-      <c r="M82" s="6">
+      <c r="M82" s="13">
         <v>5062775445863580</v>
       </c>
       <c r="N82">
@@ -4640,13 +4644,13 @@
       <c r="F83">
         <v>0</v>
       </c>
-      <c r="G83" s="13">
+      <c r="G83" s="12">
         <v>0</v>
       </c>
       <c r="H83">
         <v>0</v>
       </c>
-      <c r="I83" s="13">
+      <c r="I83" s="12">
         <v>0</v>
       </c>
       <c r="J83">
@@ -4684,13 +4688,13 @@
       <c r="F84">
         <v>0</v>
       </c>
-      <c r="G84" s="13">
+      <c r="G84" s="12">
         <v>0</v>
       </c>
       <c r="H84">
         <v>0</v>
       </c>
-      <c r="I84" s="13">
+      <c r="I84" s="12">
         <v>0</v>
       </c>
       <c r="J84">
@@ -4728,13 +4732,13 @@
       <c r="F85">
         <v>0</v>
       </c>
-      <c r="G85" s="13">
+      <c r="G85" s="12">
         <v>0</v>
       </c>
       <c r="H85">
         <v>0</v>
       </c>
-      <c r="I85" s="13">
+      <c r="I85" s="12">
         <v>0</v>
       </c>
       <c r="J85">
@@ -4772,13 +4776,13 @@
       <c r="F86">
         <v>0</v>
       </c>
-      <c r="G86" s="13">
+      <c r="G86" s="12">
         <v>0</v>
       </c>
       <c r="H86">
         <v>0</v>
       </c>
-      <c r="I86" s="13">
+      <c r="I86" s="12">
         <v>0</v>
       </c>
       <c r="J86">
@@ -4816,13 +4820,13 @@
       <c r="F87">
         <v>0</v>
       </c>
-      <c r="G87" s="13">
+      <c r="G87" s="12">
         <v>0</v>
       </c>
       <c r="H87">
         <v>0</v>
       </c>
-      <c r="I87" s="13">
+      <c r="I87" s="12">
         <v>0</v>
       </c>
       <c r="J87">
@@ -4860,13 +4864,13 @@
       <c r="F88">
         <v>0</v>
       </c>
-      <c r="G88" s="13">
+      <c r="G88" s="12">
         <v>0</v>
       </c>
       <c r="H88">
         <v>0</v>
       </c>
-      <c r="I88" s="13">
+      <c r="I88" s="12">
         <v>0</v>
       </c>
       <c r="J88">
@@ -4904,13 +4908,13 @@
       <c r="F89">
         <v>0</v>
       </c>
-      <c r="G89" s="13">
+      <c r="G89" s="12">
         <v>0</v>
       </c>
       <c r="H89">
         <v>0</v>
       </c>
-      <c r="I89" s="13">
+      <c r="I89" s="12">
         <v>0</v>
       </c>
       <c r="J89">
@@ -4948,13 +4952,13 @@
       <c r="F90">
         <v>0</v>
       </c>
-      <c r="G90" s="13">
+      <c r="G90" s="12">
         <v>0</v>
       </c>
       <c r="H90">
         <v>0</v>
       </c>
-      <c r="I90" s="13">
+      <c r="I90" s="12">
         <v>0</v>
       </c>
       <c r="J90">
@@ -4966,10 +4970,10 @@
       <c r="L90">
         <v>0</v>
       </c>
-      <c r="M90" s="13">
-        <v>0</v>
-      </c>
-      <c r="N90" s="13">
+      <c r="M90" s="12">
+        <v>0</v>
+      </c>
+      <c r="N90" s="12">
         <v>1.1865088354049E+16</v>
       </c>
     </row>
@@ -4992,13 +4996,13 @@
       <c r="F91">
         <v>0</v>
       </c>
-      <c r="G91" s="13">
+      <c r="G91" s="12">
         <v>0</v>
       </c>
       <c r="H91">
         <v>0</v>
       </c>
-      <c r="I91" s="13">
+      <c r="I91" s="12">
         <v>0</v>
       </c>
       <c r="J91">
@@ -5010,7 +5014,7 @@
       <c r="L91">
         <v>0</v>
       </c>
-      <c r="M91" s="13">
+      <c r="M91" s="12">
         <v>0</v>
       </c>
       <c r="N91">
@@ -5036,13 +5040,13 @@
       <c r="F92">
         <v>0</v>
       </c>
-      <c r="G92" s="13">
+      <c r="G92" s="12">
         <v>0</v>
       </c>
       <c r="H92">
         <v>0</v>
       </c>
-      <c r="I92" s="13">
+      <c r="I92" s="12">
         <v>0</v>
       </c>
       <c r="J92">
@@ -5054,10 +5058,10 @@
       <c r="L92">
         <v>0</v>
       </c>
-      <c r="M92" s="13">
-        <v>0</v>
-      </c>
-      <c r="N92" s="13">
+      <c r="M92" s="12">
+        <v>0</v>
+      </c>
+      <c r="N92" s="12">
         <v>1.82639924706312E+16</v>
       </c>
     </row>
@@ -45187,7 +45191,7 @@
         <v>153</v>
       </c>
       <c r="B1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -45553,7 +45557,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A1424E3-65E6-4D4E-8617-9B434C5DD01D}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -45579,6 +45583,11 @@
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>187</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
emissions updated and more user-friendly
smoking and frying emission were updated and the mod_var_setup file was made more user-friendly by adding further flags for turning off indoor activities
</commit_message>
<xml_diff>
--- a/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
+++ b/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livemanchesterac-my.sharepoint.com/personal/simon_omeara_manchester_ac_uk/Documents/GitHub/NCAS-BoxModellingToolkit/indoor_environment_PyCHAM_setup/src/indoor_environment_PyCHAM_setup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{2EF619C7-E479-174A-A447-3F7B7DC38047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12471697-6F5D-45C6-B4C4-01B84BD84897}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{2EF619C7-E479-174A-A447-3F7B7DC38047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F4AEA92-6BCF-4106-A999-19A387A4ACFD}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="120" windowWidth="16188" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="840" windowWidth="18924" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_emi" sheetId="1" r:id="rId1"/>
@@ -1136,10 +1136,10 @@
         <v>0</v>
       </c>
       <c r="E3">
-        <v>147166666666.67001</v>
+        <v>300000000000</v>
       </c>
       <c r="F3" s="13">
-        <v>3955104166666.75</v>
+        <v>2000000000000</v>
       </c>
       <c r="G3" s="8">
         <v>0</v>

</xml_diff>

<commit_message>
bug fix and emission updates
flickering candle and frying emissions have been updated. Allocation of outdoor PM to size bins has been fixed as previously some outdoor PM2.5 was being assigned to the middle size bin, whilst it had a size meaning it should have been assigned to the smallest size bin
</commit_message>
<xml_diff>
--- a/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
+++ b/src/indoor_environment_PyCHAM_setup/indoor_emi_pri_org_VBS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livemanchesterac-my.sharepoint.com/personal/simon_omeara_manchester_ac_uk/Documents/GitHub/NCAS-BoxModellingToolkit/indoor_environment_PyCHAM_setup/src/indoor_environment_PyCHAM_setup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{2EF619C7-E479-174A-A447-3F7B7DC38047}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE263203-6F97-1842-A4E5-A17C4D03D045}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="13_ncr:1_{30D5AEC0-A9C1-5C44-A108-36C9A8FF0C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63CA9033-BB42-4C43-9E1E-B82F3BCC37B7}"/>
   <bookViews>
-    <workbookView xWindow="5920" yWindow="4620" windowWidth="22780" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="60" yWindow="500" windowWidth="24280" windowHeight="12020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indoor_emi" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="208">
   <si>
     <t>ACRYLONITRILE</t>
   </si>
@@ -641,12 +641,6 @@
     <t>this paper 10.1021/es202946w (emission rates of PM2.5 (ug/min) in Table 1 gives similar values to those reported in https://doi.org/10.1016/j.buildenv.2020.107059, though notes that in certan tests the emission rate was up to 3 orders of magnitude higher), it is noted that https://doi.org/10.1016/j.buildenv.2020.107059 does not account for particle loss to indoor surfaces, therefore values were increased by a factor 2.5 to correct for this</t>
   </si>
   <si>
-    <t>Frying (these values represent particles/ or molecules/s/person/meal or mole fraction of particles; particles from 10.1016/j.atmosenv.2010.01.009, using Table 2, which gives units in /min, and so /60 to convert to /s, e.g. 8.02e12 particles/60, gases from https://onlinelibrary.wiley.com/doi/full/10.1111/ina.12906 (Table 4), assuming stir fry lasted 15 minutes, e.g. for ethanol from table 4: ((67.e-3/46.0684)*6.022e23)/(15.*60.), note that citral not in MCM, so represented by limonene).  Particle radius of 0.03 um is suggested by Figure 12 of this reference (10.1016/j.atmosenv.2010.01.009). Black carbon to primary organic mole fractions estimated from Table 18 of http://dx.doi.org/10.1016/j.atmosenv.2013.01.061</t>
-  </si>
-  <si>
-    <t>candle burning (doi.org/10.1016/j.jaerosci.2008.10.005), which shows in Fig. 10 that most particle mass is in candles with a diameter less than 160 nm, the arithmetic mean of steady burn PM2.5 mass emission factor for their candle 1 and candle 2 in Table 1 is 1.635 mg/h, which converts to 4.54e-7 g/s. Then need to convert to particles/s by dividing by the mass of one particle, and Fig 10. shows that most mass during steady burn has particle radius around 50 nm, which gives a volume of 4/3*np.pi*50e-7**3 cm^3 = 5.24e-16 cm^3, and the density is based on Table 3 that indicates that potassium nitrate is a main mass contributor to candle particles, which is supported by the internet that says potassium nitrate is used to help the wick burn, then 5.24e-16*2.11 cm^3=1.11e-15g per particle, so the particle emission rate is 4.54e-7 g/s/1.11e-15g/particle = 4.09e8 particle/s</t>
-  </si>
-  <si>
     <t>POT_NIT_ind_pm0</t>
   </si>
   <si>
@@ -658,12 +652,24 @@
   <si>
     <t>POT_NIT_ind_pm2</t>
   </si>
+  <si>
+    <t>candle burning (doi.org/10.1016/j.jaerosci.2008.10.005), which shows in Fig. 10 that most particle mass is in candles with a diameter less than 160 nm, the arithmetic mean of steady burn PM2.5 mass emission factor for their candle 1 and candle 2 in Table 1 is 1.635 mg/h, which converts to 4.54e-7 g/s. Then need to convert to particles/s by dividing by the mass of one particle, and Fig 10. shows that most mass during steady burn has particle radius around 50 nm, which gives a volume of 4/3*np.pi*50e-7**3 cm^3 = 5.24e-16 cm^3, and the density is based on Table 3 that indicates that potassium nitrate is a main mass contributor to candle particles, which is supported by the internet that says potassium nitrate is used to help the wick burn, then 5.24e-16*2.11 cm^3=1.11e-15g per particle, so the particle emission rate is 4.54e-7 g/s/1.11e-15g/particle = 4.09e8 particle/s. Note that this emission rate, and combined particle radius has been tested against the lab observations in their Fig. 6 for wall deposition of particles rates typical of chambers</t>
+  </si>
+  <si>
+    <t>dirty gas fire place, with pconc tuned to PM2.5 values seen for combustion household</t>
+  </si>
+  <si>
+    <t>Frying (these values represent particles/ or molecules/s or mole fraction of particles; particles from 10.1016/j.atmosenv.2010.01.009, where ultrafine particles have radius 50 nm or less, using Table 2, which gives units in /min, and so /60 to convert to /s, e.g. 7.66e12 particles/60=1.3e11 /s. Note that for some of the particle emission in Table 2 for frying, the number emitted has a contribution from larger than ultrafine particles. Fig 6c of https://doi.org/10.1016/j.atmosenv.2009.03.044 shows that mass peak for frying occurs around 0.3um diameter, so this determines the radius of the second size bin here. In addition, Table 6 of https://doi.org/10.1016/j.atmosenv.2009.03.044 reports a peak mass concentration of particles (which is generated at full gas stove power) of 118 ug/m3, which is reproduced by the values below in the test simulation for reproducing their experimental conditions, with inputs saved in fry_test_against_doiporgslash10p1016slashjpatmosenvp2009p03p044. Note that using a mean radius for the second size bin of 0.1 um led to quick transfer of these particles to the smaller size bin, presumably because of evaporation of volatiles. Results from testing frying inputs are saved in frying_test_doi_10p1016dashjpatmosenvp2010p01p009. Gases from https://onlinelibrary.wiley.com/doi/full/10.1111/ina.12906 (Table 4), assuming stir fry lasted 15 minutes, e.g. for ethanol from table 4: ((67.e-3/46.0684)*6.022e23)/(15.*60.), note that citral not in MCM, so represented by limonene). Black carbon to primary organic mole fractions estimated from Table 18 of http://dx.doi.org/10.1016/j.atmosenv.2013.01.061</t>
+  </si>
+  <si>
+    <t>flickering candle, from Table 2 of doi.org/10.1111/ina.12909 (Candle 5), 1.5e13/3600 =  5.17e9 particles/s are generated, whilst their Fig 2. suggests a small fraction of this number is in a larger mode. Table 2 indicates these particles are composed of elemental carbon (with a molar mass of 12.01 g/mol), Table 2 also says that 4346/3600= 1.21 ug/s of black carbon is released. Fig 2 shows that most particle mass is in the larger mode particles, so assuming 1.20 ug/s comes from the large mode and 0.01 ug/s comes from the small mode, and that of the total number emitted 0.1 % is in the larger mode, then each large mode particle must contain 1.20/(5.17e9*0.001) =  2.32e-7 ug of carbon. Carbon as graphite has a density of 2.26 g/cm^3, which means each particle has a volume 2.32e-13 g/particle/2.26 g/cm^3 = 1.03e-13 cm^3, which is a radius of (V*3/(4.*np.pi))**(1./3.) 2.91e-5 cm, which is 0.291 um. Using the same template for the smaller particles gives ((0.01/(5.17e9*0.999)*1.e-6/2.26*3.)/(4.*np.pi))**(1./3.)=5.89e-7cm or 0.00589 um. However, this value for the larger particles does not get anywhere near the mass concentrations of PM2.5 seen in the combustion household of INGENIOUS. Instead, the mean radius was set to 0.45 um, which is consistent with the Candle 5 plot of mass-size distribution in Fig.2 of  https://doi.org/10.1111/ina.12909, whilst the number concentration was tuned to give emission factors of PM2.5 consistent with Table 1 of https://doi.org/10.1016/j.envint.2011.07.009, which report possible emisssion factors from candles of 15 mg/g. Table 2 of https://doi.org/10.1111/ina.12909 shows a typical burn rate of 5g/hour for candles, so one can do the calculation: 15.(mg/g)*1.e3(mg to ug)*5.(g/hr)/3600(per hr to per s) = 21 ug/s, whilst the values used here give a rate of (4./3.)*np.pi*0.45e-4**3(cm^3/particle)*2.26(g/cm^3)*1.e6(g/particle to ug/particle)*25850000(particles/s)=22 ug/s. This value is the same order of magnitude as reported in Table 1 for candle II of https://doi.org/10.1016/j.jaerosci.2008.10.005, which reports that during sooting (flickering), mass emission rates can be around 25 mg/hour, which equates to 25*1.e3(mg to ug)/3600(hour to s) = 7 ug/s, which is also the mass emission factor reported from a real home in Table 2 of https://doi.org/10.1016/j.buildenv.2021.108422</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -691,6 +697,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Menlo"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -734,7 +746,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -764,10 +776,11 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1055,7 +1068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P10121"/>
+  <dimension ref="A1:R10121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.5" customWidth="1"/>
@@ -1063,7 +1076,7 @@
     <col min="3" max="3" width="32.1640625" style="4" customWidth="1"/>
     <col min="4" max="4" width="29" style="4" customWidth="1"/>
     <col min="5" max="5" width="32.1640625" customWidth="1"/>
-    <col min="6" max="6" width="22.33203125" customWidth="1"/>
+    <col min="6" max="6" width="35.6640625" customWidth="1"/>
     <col min="7" max="7" width="19.5" customWidth="1"/>
     <col min="8" max="8" width="19.6640625" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
@@ -1072,22 +1085,25 @@
     <col min="12" max="12" width="15.1640625" customWidth="1"/>
     <col min="13" max="13" width="16.33203125" customWidth="1"/>
     <col min="14" max="14" width="12.6640625" customWidth="1"/>
+    <col min="15" max="15" width="18.6640625" customWidth="1"/>
+    <col min="16" max="16" width="14" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="7"/>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="17" t="s">
         <v>160</v>
       </c>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
       <c r="I1" s="8"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>21</v>
       </c>
@@ -1104,7 +1120,7 @@
         <v>185</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>136</v>
@@ -1134,10 +1150,16 @@
         <v>155</v>
       </c>
       <c r="P2" s="8" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+        <v>204</v>
+      </c>
+      <c r="Q2" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="R2" s="8" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
         <v>53</v>
       </c>
@@ -1153,8 +1175,8 @@
       <c r="E3">
         <v>300000000000</v>
       </c>
-      <c r="F3" s="13">
-        <v>2000000000000</v>
+      <c r="F3" s="16">
+        <v>129666666666.666</v>
       </c>
       <c r="G3" s="8">
         <v>0</v>
@@ -1184,10 +1206,16 @@
         <v>0</v>
       </c>
       <c r="P3" s="16">
-        <v>409000000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+        <v>400000000</v>
+      </c>
+      <c r="Q3" s="16">
+        <v>5164830000</v>
+      </c>
+      <c r="R3" s="15">
+        <v>1200000000000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
@@ -1236,8 +1264,14 @@
       <c r="P4" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q4" s="16">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>149</v>
       </c>
@@ -1286,8 +1320,14 @@
       <c r="P5" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q5" s="16">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>143</v>
       </c>
@@ -1336,8 +1376,14 @@
       <c r="P6" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q6" s="16">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>158</v>
       </c>
@@ -1386,13 +1432,19 @@
       <c r="P7" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q7" s="16">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C8">
         <v>101.1</v>
@@ -1436,8 +1488,14 @@
       <c r="P8" s="8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q8" s="16">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>83</v>
       </c>
@@ -1484,8 +1542,14 @@
       <c r="P9" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q9" s="16">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>80</v>
       </c>
@@ -1532,8 +1596,14 @@
       <c r="P10" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q10" s="16">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>84</v>
       </c>
@@ -1580,8 +1650,14 @@
       <c r="P11" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q11" s="16">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>94</v>
       </c>
@@ -1628,8 +1704,14 @@
       <c r="P12" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q12" s="16">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>62</v>
       </c>
@@ -1675,8 +1757,14 @@
       <c r="P13" s="8">
         <v>0.05</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q13" s="16">
+        <v>5.8900000000000003E-3</v>
+      </c>
+      <c r="R13">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
         <v>52</v>
       </c>
@@ -1692,8 +1780,8 @@
       <c r="E14">
         <v>0</v>
       </c>
-      <c r="F14">
-        <v>0</v>
+      <c r="F14" s="16">
+        <v>4000000000</v>
       </c>
       <c r="G14" s="8">
         <v>0</v>
@@ -1722,11 +1810,17 @@
       <c r="O14" s="8">
         <v>0</v>
       </c>
-      <c r="P14" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="P14" s="16">
+        <v>9000000</v>
+      </c>
+      <c r="Q14" s="16">
+        <v>25850000</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>65</v>
       </c>
@@ -1743,7 +1837,7 @@
         <v>0</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>9.0899999999999995E-2</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -1775,8 +1869,14 @@
       <c r="P15" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q15" s="16">
+        <v>1</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>151</v>
       </c>
@@ -1825,8 +1925,14 @@
       <c r="P16" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q16" s="16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>144</v>
       </c>
@@ -1875,8 +1981,14 @@
       <c r="P17" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q17" s="16">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>159</v>
       </c>
@@ -1925,13 +2037,19 @@
       <c r="P18" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q18" s="16">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C19">
         <v>101.1</v>
@@ -1973,10 +2091,16 @@
         <v>0</v>
       </c>
       <c r="P19" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="16">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>82</v>
       </c>
@@ -2023,8 +2147,14 @@
       <c r="P20" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q20" s="16">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>81</v>
       </c>
@@ -2039,7 +2169,7 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>0.18634239288307916</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -2071,8 +2201,14 @@
       <c r="P21" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q21" s="16">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>85</v>
       </c>
@@ -2087,7 +2223,7 @@
         <v>0</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>0.39348119099491646</v>
       </c>
       <c r="G22">
         <v>0</v>
@@ -2119,8 +2255,14 @@
       <c r="P22" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q22" s="16">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>86</v>
       </c>
@@ -2135,7 +2277,7 @@
         <v>0</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>0.32927641612200437</v>
       </c>
       <c r="G23">
         <v>0</v>
@@ -2167,8 +2309,14 @@
       <c r="P23" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q23" s="16">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>63</v>
       </c>
@@ -2182,7 +2330,7 @@
         <v>0</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="G24">
         <v>0</v>
@@ -2212,10 +2360,16 @@
         <v>0</v>
       </c>
       <c r="P24" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
+        <v>0.2</v>
+      </c>
+      <c r="Q24" s="16">
+        <v>0.45</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>189</v>
       </c>
@@ -2264,8 +2418,14 @@
       <c r="P25" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q25" s="16">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" s="11" t="s">
         <v>190</v>
       </c>
@@ -2314,8 +2474,14 @@
       <c r="P26" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q26" s="16">
+        <v>0</v>
+      </c>
+      <c r="R26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>191</v>
       </c>
@@ -2364,8 +2530,14 @@
       <c r="P27" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q27" s="16">
+        <v>0</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>192</v>
       </c>
@@ -2414,8 +2586,14 @@
       <c r="P28" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q28" s="16">
+        <v>0</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>193</v>
       </c>
@@ -2464,13 +2642,19 @@
       <c r="P29" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q29" s="16">
+        <v>0</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C30" s="4">
         <v>0</v>
@@ -2514,8 +2698,14 @@
       <c r="P30" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q30" s="16">
+        <v>0</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>194</v>
       </c>
@@ -2562,8 +2752,14 @@
       <c r="P31" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q31" s="16">
+        <v>0</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>195</v>
       </c>
@@ -2610,8 +2806,14 @@
       <c r="P32" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q32" s="16">
+        <v>0</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>196</v>
       </c>
@@ -2658,8 +2860,14 @@
       <c r="P33" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q33" s="16">
+        <v>0</v>
+      </c>
+      <c r="R33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>197</v>
       </c>
@@ -2706,8 +2914,14 @@
       <c r="P34" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q34" s="16">
+        <v>0</v>
+      </c>
+      <c r="R34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>198</v>
       </c>
@@ -2753,8 +2967,14 @@
       <c r="P35" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q35" s="16">
+        <v>0</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>54</v>
       </c>
@@ -2803,8 +3023,14 @@
       <c r="P36" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q36" s="16">
+        <v>0</v>
+      </c>
+      <c r="R36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
         <v>38</v>
       </c>
@@ -2853,8 +3079,14 @@
       <c r="P37" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q37" s="16">
+        <v>0</v>
+      </c>
+      <c r="R37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>40</v>
       </c>
@@ -2903,8 +3135,14 @@
       <c r="P38" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q38" s="16">
+        <v>0</v>
+      </c>
+      <c r="R38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>23</v>
       </c>
@@ -2953,8 +3191,14 @@
       <c r="P39" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q39" s="16">
+        <v>0</v>
+      </c>
+      <c r="R39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>25</v>
       </c>
@@ -3003,8 +3247,14 @@
       <c r="P40" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q40" s="16">
+        <v>0</v>
+      </c>
+      <c r="R40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>27</v>
       </c>
@@ -3053,8 +3303,14 @@
       <c r="P41" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q41" s="16">
+        <v>0</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>29</v>
       </c>
@@ -3103,8 +3359,14 @@
       <c r="P42" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q42" s="16">
+        <v>0</v>
+      </c>
+      <c r="R42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>31</v>
       </c>
@@ -3153,8 +3415,14 @@
       <c r="P43" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q43" s="16">
+        <v>0</v>
+      </c>
+      <c r="R43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>36</v>
       </c>
@@ -3203,8 +3471,14 @@
       <c r="P44" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q44" s="16">
+        <v>0</v>
+      </c>
+      <c r="R44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
         <v>11</v>
       </c>
@@ -3253,8 +3527,14 @@
       <c r="P45" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q45" s="16">
+        <v>0</v>
+      </c>
+      <c r="R45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>12</v>
       </c>
@@ -3303,8 +3583,14 @@
       <c r="P46" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q46" s="16">
+        <v>0</v>
+      </c>
+      <c r="R46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
         <v>13</v>
       </c>
@@ -3353,8 +3639,14 @@
       <c r="P47" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q47" s="16">
+        <v>0</v>
+      </c>
+      <c r="R47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>0</v>
       </c>
@@ -3403,8 +3695,14 @@
       <c r="P48" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q48" s="16">
+        <v>0</v>
+      </c>
+      <c r="R48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>14</v>
       </c>
@@ -3453,8 +3751,14 @@
       <c r="P49" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q49" s="16">
+        <v>0</v>
+      </c>
+      <c r="R49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>2</v>
       </c>
@@ -3503,8 +3807,14 @@
       <c r="P50" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q50" s="16">
+        <v>0</v>
+      </c>
+      <c r="R50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>1</v>
       </c>
@@ -3553,8 +3863,14 @@
       <c r="P51" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q51" s="16">
+        <v>0</v>
+      </c>
+      <c r="R51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>3</v>
       </c>
@@ -3603,8 +3919,14 @@
       <c r="P52" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q52" s="16">
+        <v>0</v>
+      </c>
+      <c r="R52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>20</v>
       </c>
@@ -3653,8 +3975,14 @@
       <c r="P53" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q53" s="16">
+        <v>0</v>
+      </c>
+      <c r="R53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>15</v>
       </c>
@@ -3703,8 +4031,14 @@
       <c r="P54" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q54" s="16">
+        <v>0</v>
+      </c>
+      <c r="R54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
         <v>16</v>
       </c>
@@ -3753,8 +4087,14 @@
       <c r="P55" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q55" s="16">
+        <v>0</v>
+      </c>
+      <c r="R55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>4</v>
       </c>
@@ -3803,8 +4143,14 @@
       <c r="P56" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q56" s="16">
+        <v>0</v>
+      </c>
+      <c r="R56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -3853,8 +4199,14 @@
       <c r="P57" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q57" s="16">
+        <v>0</v>
+      </c>
+      <c r="R57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>5</v>
       </c>
@@ -3903,8 +4255,14 @@
       <c r="P58" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q58" s="16">
+        <v>0</v>
+      </c>
+      <c r="R58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
         <v>57</v>
       </c>
@@ -3953,8 +4311,14 @@
       <c r="P59" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q59" s="16">
+        <v>0</v>
+      </c>
+      <c r="R59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>58</v>
       </c>
@@ -4003,8 +4367,14 @@
       <c r="P60" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q60" s="16">
+        <v>0</v>
+      </c>
+      <c r="R60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>6</v>
       </c>
@@ -4053,8 +4423,14 @@
       <c r="P61" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q61" s="16">
+        <v>0</v>
+      </c>
+      <c r="R61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
         <v>18</v>
       </c>
@@ -4103,8 +4479,14 @@
       <c r="P62" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q62" s="16">
+        <v>0</v>
+      </c>
+      <c r="R62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
         <v>18</v>
       </c>
@@ -4153,8 +4535,14 @@
       <c r="P63" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q63" s="16">
+        <v>0</v>
+      </c>
+      <c r="R63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>7</v>
       </c>
@@ -4203,8 +4591,14 @@
       <c r="P64" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q64" s="16">
+        <v>0</v>
+      </c>
+      <c r="R64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>59</v>
       </c>
@@ -4253,8 +4647,14 @@
       <c r="P65" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q65" s="16">
+        <v>0</v>
+      </c>
+      <c r="R65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>60</v>
       </c>
@@ -4303,8 +4703,14 @@
       <c r="P66" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q66" s="16">
+        <v>0</v>
+      </c>
+      <c r="R66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>8</v>
       </c>
@@ -4353,8 +4759,14 @@
       <c r="P67" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q67" s="16">
+        <v>0</v>
+      </c>
+      <c r="R67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>61</v>
       </c>
@@ -4403,8 +4815,14 @@
       <c r="P68" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q68" s="16">
+        <v>0</v>
+      </c>
+      <c r="R68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
         <v>9</v>
       </c>
@@ -4453,8 +4871,14 @@
       <c r="P69" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q69" s="16">
+        <v>0</v>
+      </c>
+      <c r="R69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
         <v>10</v>
       </c>
@@ -4503,8 +4927,14 @@
       <c r="P70" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q70" s="16">
+        <v>0</v>
+      </c>
+      <c r="R70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
         <v>33</v>
       </c>
@@ -4553,8 +4983,14 @@
       <c r="P71" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q71" s="16">
+        <v>0</v>
+      </c>
+      <c r="R71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
         <v>42</v>
       </c>
@@ -4603,8 +5039,14 @@
       <c r="P72" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q72" s="16">
+        <v>0</v>
+      </c>
+      <c r="R72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
         <v>44</v>
       </c>
@@ -4653,8 +5095,14 @@
       <c r="P73" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q73" s="16">
+        <v>0</v>
+      </c>
+      <c r="R73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>46</v>
       </c>
@@ -4703,8 +5151,14 @@
       <c r="P74" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q74" s="16">
+        <v>0</v>
+      </c>
+      <c r="R74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>48</v>
       </c>
@@ -4753,8 +5207,14 @@
       <c r="P75" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q75" s="16">
+        <v>0</v>
+      </c>
+      <c r="R75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
         <v>50</v>
       </c>
@@ -4803,8 +5263,14 @@
       <c r="P76" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q76" s="16">
+        <v>0</v>
+      </c>
+      <c r="R76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
         <v>96</v>
       </c>
@@ -4853,8 +5319,14 @@
       <c r="P77" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q77" s="16">
+        <v>0</v>
+      </c>
+      <c r="R77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>98</v>
       </c>
@@ -4903,8 +5375,14 @@
       <c r="P78" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q78" s="16">
+        <v>0</v>
+      </c>
+      <c r="R78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>101</v>
       </c>
@@ -4953,8 +5431,14 @@
       <c r="P79" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q79" s="16">
+        <v>0</v>
+      </c>
+      <c r="R79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>103</v>
       </c>
@@ -5003,8 +5487,14 @@
       <c r="P80" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q80" s="16">
+        <v>0</v>
+      </c>
+      <c r="R80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
         <v>105</v>
       </c>
@@ -5053,8 +5543,14 @@
       <c r="P81" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q81" s="16">
+        <v>0</v>
+      </c>
+      <c r="R81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>107</v>
       </c>
@@ -5103,8 +5599,14 @@
       <c r="P82" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q82" s="16">
+        <v>0</v>
+      </c>
+      <c r="R82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>108</v>
       </c>
@@ -5153,8 +5655,14 @@
       <c r="P83" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q83" s="16">
+        <v>0</v>
+      </c>
+      <c r="R83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
         <v>110</v>
       </c>
@@ -5203,8 +5711,14 @@
       <c r="P84" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q84" s="16">
+        <v>0</v>
+      </c>
+      <c r="R84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
         <v>176</v>
       </c>
@@ -5253,8 +5767,14 @@
       <c r="P85" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q85" s="16">
+        <v>0</v>
+      </c>
+      <c r="R85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
         <v>175</v>
       </c>
@@ -5303,8 +5823,14 @@
       <c r="P86" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q86" s="16">
+        <v>0</v>
+      </c>
+      <c r="R86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
         <v>174</v>
       </c>
@@ -5353,8 +5879,14 @@
       <c r="P87" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q87" s="16">
+        <v>0</v>
+      </c>
+      <c r="R87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>164</v>
       </c>
@@ -5403,8 +5935,14 @@
       <c r="P88" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q88" s="16">
+        <v>0</v>
+      </c>
+      <c r="R88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
         <v>166</v>
       </c>
@@ -5453,8 +5991,14 @@
       <c r="P89" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q89" s="16">
+        <v>0</v>
+      </c>
+      <c r="R89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
         <v>168</v>
       </c>
@@ -5503,8 +6047,14 @@
       <c r="P90" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q90" s="16">
+        <v>0</v>
+      </c>
+      <c r="R90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
         <v>170</v>
       </c>
@@ -5553,8 +6103,14 @@
       <c r="P91" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q91" s="16">
+        <v>0</v>
+      </c>
+      <c r="R91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
         <v>172</v>
       </c>
@@ -5603,8 +6159,14 @@
       <c r="P92" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q92" s="16">
+        <v>0</v>
+      </c>
+      <c r="R92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>177</v>
       </c>
@@ -5653,8 +6215,14 @@
       <c r="P93" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q93" s="16">
+        <v>0</v>
+      </c>
+      <c r="R93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>180</v>
       </c>
@@ -5703,8 +6271,14 @@
       <c r="P94" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q94" s="16">
+        <v>0</v>
+      </c>
+      <c r="R94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>182</v>
       </c>
@@ -5753,8 +6327,14 @@
       <c r="P95" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q95" s="16">
+        <v>0</v>
+      </c>
+      <c r="R95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
     </row>

</xml_diff>